<commit_message>
台帳と xlsx に KAKUSEI・KOUSEN を追加
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011CXCQ6yZPAA1DkPDCtnjdd
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1916,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3562,12 +3562,12 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>MADOKAGAMI</t>
+          <t>KAKUSEI</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>カメラに映った顔と手が小さなアプリのウィンドウの群れに分解されるエフェクト。窓の中身はいまの映像そのもので動けば群れがついてくる。背景は青空と丘のデスクトップ壁紙で手を掲げるほど窓が増える。</t>
+          <t>映った人がアニメのセル画になり体から気のオーラが燃え上がるエフェクト。声を出すほど炎が大きくなり叫びきると一瞬だけ白黒反転の決めカットになる。録画して保存できる。</t>
         </is>
       </c>
       <c r="F53" s="6" t="n"/>
@@ -3588,17 +3588,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>ZANZOU</t>
+          <t>KOUSEN</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>カメラに映った人物だけを白黒のクロスハッチ線画にするエフェクト。動いた跡は青・マゼンタ・黄の色つきシルエットになって遅れてついてくる。線の細かさ・遅れ・コントラスト・配色を操作パネルで調整できる。</t>
+          <t>暗いステージに立つと床とトラスのレーザーがあなたの輪郭をなぞりつづけるエフェクト。体は逆光のライブ写真のような二色になり手を叩くたびにストロボが焚かれて照明が切り替わる。録画して保存できる。</t>
         </is>
       </c>
       <c r="F54" s="6" t="n"/>
@@ -3619,17 +3619,17 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>KORIN</t>
+          <t>MADOKAGAMI</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>カメラに映った顔にタンバリンの光輪をかぶったバケットハットが天から落ちて乗るエフェクト。頭を傾ければ帽子も傾き着地の瞬間に本物のジングルが鳴る。画面いっぱいの表示で調整パネルは引っ込められ録画すればその音ごと保存できる。</t>
+          <t>カメラに映った顔と手が小さなアプリのウィンドウの群れに分解されるエフェクト。窓の中身はいまの映像そのもので動けば群れがついてくる。背景は青空と丘のデスクトップ壁紙で手を掲げるほど窓が増える。</t>
         </is>
       </c>
       <c r="F55" s="6" t="n"/>
@@ -3639,10 +3639,72 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>ZANZOU</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>カメラに映った人物だけを白黒のクロスハッチ線画にするエフェクト。動いた跡は青・マゼンタ・黄の色つきシルエットになって遅れてついてくる。線の細かさ・遅れ・コントラスト・配色を操作パネルで調整できる。</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>KORIN</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>カメラに映った顔にタンバリンの光輪をかぶったバケットハットが天から落ちて乗るエフェクト。頭を傾ければ帽子も傾き着地の瞬間に本物のジングルが鳴る。画面いっぱいの表示で調整パネルは引っ込められ録画すればその音ごと保存できる。</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n"/>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G55"/>
+  <autoFilter ref="A1:G57"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3701,6 +3763,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -3847,7 +3911,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$55,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$57,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -3870,7 +3934,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$55,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$57,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -3893,7 +3957,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$55,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$57,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -3914,7 +3978,7 @@
         <v>22</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
HABATAKI: a film-poster double exposure whose outline flies off as birds
The person becomes a silhouette filled with a misty pine forest and a
red sun, face on top; wherever the silhouette moves, its edge peels
away into a flock of ink birds. Starts as the plain camera and switches
with a burn-out-and-develop transition. Card, works.csv, xlsx, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NAomKCCP1pC7Pkj22gVg2Q
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1143,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1874,10 +1874,41 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>BAKUON</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>体の動きがそのまま歪んだノイズシンセになる。音色を作っているのはあなたの姿を縦に切った一本の線。高いところで動けば高く暴れるほど七つの発振器が折れて唸り太鼓が組み上がる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>楽器</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G23"/>
+  <autoFilter ref="A1:G24"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1904,6 +1935,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -1916,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4027,12 +4059,12 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>HAIKOU</t>
+          <t>DANSEN</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>頭のうしろに強い光が灯りあなたは黒い影になって輪郭のすきまから光の筋が霧へ噴き出す。止まれば静かな後光動くほど光芒は長く激しくなる。</t>
+          <t>カメラに映るものが割れた液晶に映った像になる。動いたところの配線から死んで純色の縦線が画面を貫き帯になった行は像を横へ引き伸ばす。壊れた跡は消えず画面をタップすると罅が走る。</t>
         </is>
       </c>
       <c r="F68" s="6" t="n"/>
@@ -4058,12 +4090,12 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>RINBU</t>
+          <t>HAIKOU</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>切り抜かれたあなたが八人に増え紙の上で万華鏡の花になる。一人ずつ少し遅れているので動けば波が輪を一周し花は回り出して朱の刷り跡を残す。止まれば紋章に戻る。</t>
+          <t>頭のうしろに強い光が灯りあなたは黒い影になって輪郭のすきまから光の筋が霧へ噴き出す。止まれば静かな後光動くほど光芒は長く激しくなる。</t>
         </is>
       </c>
       <c r="F69" s="6" t="n"/>
@@ -4073,10 +4105,103 @@
         </is>
       </c>
     </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>RINBU</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>切り抜かれたあなたが八人に増え紙の上で万華鏡の花になる。一人ずつ少し遅れているので動けば波が輪を一周し花は回り出して朱の刷り跡を残す。止まれば紋章に戻る。</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>TAMAYURA</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>暗い舞台で自分だけが白く照らされ動いたぶんだけ真っ赤な残像がその場に置いていかれる。残像は少し留まってから点の格子に崩れ赤い球になってこぼれ落ちて消える。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>HABATAKI</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>映った人が映画ポスターのような二重露光になりシルエットの中に霧の森と赤い太陽が写る。動いたところから輪郭が黒い鳥の群れになって飛び立つ。はじめは普通のカメラでボタンを押すと白く飛んで像が現像されるように現れる。</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="n"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G69"/>
+  <autoFilter ref="A1:G72"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4149,6 +4274,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4291,11 +4419,11 @@
         <v/>
       </c>
       <c r="C15" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$23,"〇")</f>
+        <f>COUNTIF(楽器!$B$2:$B$24,"〇")</f>
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$69,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$72,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4314,11 +4442,11 @@
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$23,"△")</f>
+        <f>COUNTIF(楽器!$B$2:$B$24,"△")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$69,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$72,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4337,11 +4465,11 @@
         <v/>
       </c>
       <c r="C17" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$23,"×")</f>
+        <f>COUNTIF(楽器!$B$2:$B$24,"×")</f>
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$69,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$72,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4359,10 +4487,10 @@
         <v>14</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KAGAMIDAMA: the person as a mirror ball that throws light round the room
Lights drop and the body becomes silver tiles; facets glint under two
orbiting spots and every tile throws a speck onto the dark room. Standing
still it turns slowly; moving spins it up so the specks streak. Starts as
the plain camera. Card, works.csv, xlsx, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NAomKCCP1pC7Pkj22gVg2Q
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4198,10 +4198,41 @@
         </is>
       </c>
     </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>KAGAMIDAMA</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>明かりが落ちて映った人が銀のタイルのミラーボールになり部屋じゅうに光の粒が散る。止まればゆっくり回り動くほど速く回って光が尾を引いて流れる。はじめは普通のカメラでボタンを押すと暗転してタイルが貼られていく。</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G72"/>
+  <autoFilter ref="A1:G73"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4277,6 +4308,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4423,7 +4455,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$72,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$73,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4446,7 +4478,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$72,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$73,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4469,7 +4501,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$72,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$73,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4490,7 +4522,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
HANTEN: the person as a flip-disc mirror that clatters where you move
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NQ9zjRV4dgCnf7TwHAev4G
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4229,10 +4229,41 @@
         </is>
       </c>
     </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>HANTEN</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>映った人が何千枚もの円盤を裏返して描くフリップディスクの鏡になる。動いたところは円盤がカチカチ鳴りながら裏返りつづけタップすると白黒の反転が波になって盤を渡る。はじめは普通のカメラでボタンを押すと斜めの波があなたを描き出す。</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="n"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G73"/>
+  <autoFilter ref="A1:G74"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4309,6 +4340,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4455,7 +4487,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$73,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$74,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4478,7 +4510,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$73,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$74,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4501,7 +4533,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$73,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$74,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4522,7 +4554,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KEHAI: the person as an aura photograph whose fog runs hot where you move
Also rejects an all-NaN segmentation mask in HANTEN instead of treating it as an empty frame.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NQ9zjRV4dgCnf7TwHAev4G
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4260,10 +4260,41 @@
         </is>
       </c>
     </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>KEHAI</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>映った人がインスタント写真のオーラ写真になり暗がりの中で体のまわりに色の霧が立ちのぼる。止まっていれば静かな藍で動いたところからは熱い色の煙が噴き出し体の動いた向きへ尾を引いて渦を巻く。はじめは普通のカメラでボタンを押すと写真が現像されるように現れる。</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G74"/>
+  <autoFilter ref="A1:G75"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4341,6 +4372,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4487,7 +4519,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$74,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$75,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4510,7 +4542,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$74,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$75,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4533,7 +4565,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$74,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$75,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4554,7 +4586,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
HAGOROMO: silver monochrome figure with crimson silk flowing from the wrists
Starts as the plain camera; the switch drains the colour, darkens the room
and unfurls three Verlet silk ribbons (a buoyant shawl arcing behind the head
and two wrist tails). Faster arms lengthen the silk. Card, works.csv,
register and xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4276,12 +4276,12 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>KEHAI</t>
+          <t>KASANE</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>映った人がインスタント写真のオーラ写真になり暗がりの中で体のまわりに色の霧が立ちのぼる。止まっていれば静かな藍で動いたところからは熱い色の煙が噴き出し体の動いた向きへ尾を引いて渦を巻く。はじめは普通のカメラでボタンを押すと写真が現像されるように現れる。</t>
+          <t>映った人が何十枚もの板を重ねた等高線の彫刻になる。上の板ほど今のあなたで下の板ほど少し前のあなたなので動くと板がずれて体の軌跡が階段のように重なる。AUTOにすると動くほど色と枚数と切り口と高さが自動で変わる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F75" s="6" t="n"/>
@@ -4291,10 +4291,165 @@
         </is>
       </c>
     </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>KEHAI</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>映った人がインスタント写真のオーラ写真になり暗がりの中で体のまわりに色の霧が立ちのぼる。止まっていれば静かな藍で動いたところからは熱い色の煙が噴き出し体の動いた向きへ尾を引いて渦を巻く。はじめは普通のカメラでボタンを押すと写真が現像されるように現れる。</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>KEISEN</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>映った人が横に走る何十本もの線でできた立体になる。回すと体の裏の線は隠れ動いたところの線が波形のように震える。AUTOにすると動くほど色と線の太さと本数と奥行きが自動で変わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>KENZAN</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>映った人が針の板から押し出されたピンアートの立体になる。数千本の角柱が光を受けて浮かび動いたところの針はばねのように跳ねる。AUTOにすると動くほど色と針の太さと本数と奥行きが自動で変わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="n"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>KIRIKO</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>映った人が切子ガラスのような多面体の彫像になる。面ごとに光を受けてきらめき動いたところの面は破片になって手前へ砕け散る。AUTOにすると動くほど色と面の細かさと稜線の太さと奥行きが自動で変わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>HAGOROMO</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>映った人が黒い空間に立つ銀色のモノクロになり両手から深紅の絹が流れ出す。一枚は背中を回って頭の後ろに弧を描き腕を速く振るほど布は長く伸びて大きく翻る。はじめは普通のカメラでボタンを押すと色が抜けて布が手からほどける。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G75"/>
+  <autoFilter ref="A1:G80"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4373,6 +4528,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4519,7 +4679,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$75,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$80,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4542,7 +4702,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$75,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$80,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4565,7 +4725,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$75,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$80,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4586,7 +4746,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KIRIBARI: the camera as a Hockney-style photo joiner
Dozens of overlapping, tilted prints each re-shoot on their own clock:
stillness reads as one picture, movement splits the body across moments
and knocks prints askew. Small prints gather on the face and where you
move. Starts as the plain camera; the switch fires one shutter flash.
Card, works.csv, register and xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4446,10 +4446,41 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>KIRIBARI</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>カメラの画面が何十枚もの写真を壁に貼り合わせたコラージュになる。写真は一枚ずつ別の瞬間に撮り直されるので止まれば一枚の絵に揃い動くとあなたの体がばらばらの時刻に割れて写真が揺れる。はじめは普通のカメラでボタンを押すとシャッターが光って映像が写真の束に割れる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="n"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G80"/>
+  <autoFilter ref="A1:G81"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4533,6 +4564,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4679,7 +4711,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$80,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$81,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4702,7 +4734,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$80,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$81,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4725,7 +4757,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$80,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$81,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4746,7 +4778,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
ZUKEI: a Bauhaus poster portrait built from quarter circles and squares
Darkness picks the shape, the brightness gradient and the silhouette edge
pick its facing, and motion kicks cells round by 90° in vermilion before
they settle back. Starts as the plain camera; paper cells wipe over it.
Card, works.csv, register and xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4477,10 +4477,41 @@
         </is>
       </c>
     </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>ZUKEI</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="n"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G81"/>
+  <autoFilter ref="A1:G82"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4565,6 +4596,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4711,7 +4743,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$81,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$82,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4734,7 +4766,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$81,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$82,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4757,7 +4789,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$81,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$82,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4778,7 +4810,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
MABOROSHI: the person as a projected hologram that tears when they move
One fragment shader: dark room, a projector cone from the floor, the
masked person rebuilt from luminance with scanlines, rim light and split
colour. Rows where the body moved tear sideways in bands, and a lagging
snapshot trails as a ghost. Tap drops the signal and rebuilds it. Starts
as the plain camera. Card, works.csv, register and xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4493,12 +4493,12 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>ZUKEI</t>
+          <t>MABOROSHI</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+          <t>部屋が暗くなり映った人が床から投影されたホログラムになる。走査線と輪郭の光で透けて立ち速く動いたところから信号が裂けて横にずれ少し前の自分の残像が遅れてついてくる。はじめは普通のカメラでボタンを押すと暗転して像が床から一行ずつ組み上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F82" s="6" t="n"/>
@@ -4508,10 +4508,41 @@
         </is>
       </c>
     </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>ZUKEI</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="n"/>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G82"/>
+  <autoFilter ref="A1:G83"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4597,6 +4628,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4743,7 +4775,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$82,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$83,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4766,7 +4798,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$82,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$83,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4789,7 +4821,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$82,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$83,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4810,7 +4842,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
HAMON: contour rings in the shape of the body pour outward
Each emitted ring is an exact Euclidean distance field of the person mask
at that moment, stored in a 24-layer texture array; the shader draws a line
where distance equals age times speed. Stillness emits about one ring a
second, motion up to ten, accented. Starts as the plain camera. Card,
works.csv, register and xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4462,12 +4462,12 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>KIRIBARI</t>
+          <t>HAMON</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>カメラの画面が何十枚もの写真を壁に貼り合わせたコラージュになる。写真は一枚ずつ別の瞬間に撮り直されるので止まれば一枚の絵に揃い動くとあなたの体がばらばらの時刻に割れて写真が揺れる。はじめは普通のカメラでボタンを押すとシャッターが光って映像が写真の束に割れる。撮影と録画ができる。</t>
+          <t>映った人の輪郭からその瞬間の自分の形をした線が波紋のように広がっていく。止まっていればゆっくり一本ずつ動けばゆがんだ輪がいくつも重なってあふれ出し動いた瞬間の輪だけが差し色になる。はじめは普通のカメラでボタンを押すと暗転して体から三重の輪が放たれる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F81" s="6" t="n"/>
@@ -4493,12 +4493,12 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>MABOROSHI</t>
+          <t>KIRIBARI</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>部屋が暗くなり映った人が床から投影されたホログラムになる。走査線と輪郭の光で透けて立ち速く動いたところから信号が裂けて横にずれ少し前の自分の残像が遅れてついてくる。はじめは普通のカメラでボタンを押すと暗転して像が床から一行ずつ組み上がる。撮影と録画ができる。</t>
+          <t>カメラの画面が何十枚もの写真を壁に貼り合わせたコラージュになる。写真は一枚ずつ別の瞬間に撮り直されるので止まれば一枚の絵に揃い動くとあなたの体がばらばらの時刻に割れて写真が揺れる。はじめは普通のカメラでボタンを押すとシャッターが光って映像が写真の束に割れる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F82" s="6" t="n"/>
@@ -4524,12 +4524,12 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>ZUKEI</t>
+          <t>MABOROSHI</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+          <t>部屋が暗くなり映った人が床から投影されたホログラムになる。走査線と輪郭の光で透けて立ち速く動いたところから信号が裂けて横にずれ少し前の自分の残像が遅れてついてくる。はじめは普通のカメラでボタンを押すと暗転して像が床から一行ずつ組み上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F83" s="6" t="n"/>
@@ -4539,10 +4539,41 @@
         </is>
       </c>
     </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>ZUKEI</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="n"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G83"/>
+  <autoFilter ref="A1:G84"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4629,6 +4660,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4775,7 +4807,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$83,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$84,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4798,7 +4830,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$83,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$84,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4821,7 +4853,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$83,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$84,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4842,7 +4874,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
HARUKA: the person set before a far cinematic landscape with head parallax
Five painted layers (sky, moon or sun, far/mid ridge, near ground) are
composited with offsets proportional to the head position taken from the
mask, so the world behind shifts with true parallax. The person is re-lit
in the scene's light with a rim toward the moon or sun. Three scenes, tap
to change. Starts as the plain camera. Card, works.csv, register and xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4493,12 +4493,12 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>KIRIBARI</t>
+          <t>HARUKA</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>カメラの画面が何十枚もの写真を壁に貼り合わせたコラージュになる。写真は一枚ずつ別の瞬間に撮り直されるので止まれば一枚の絵に揃い動くとあなたの体がばらばらの時刻に割れて写真が揺れる。はじめは普通のカメラでボタンを押すとシャッターが光って映像が写真の束に割れる。撮影と録画ができる。</t>
+          <t>部屋が消えて映った人だけが映画のポスターのような遠い景色の前に立つ。大きな月と山並み・夕暮れの砂丘・霧の森。頭を動かすと景色が奥行きのとおりにずれて窓の向こうに本当に世界があるように見える。はじめは普通のカメラでボタンを押すと景色が下から順にせり上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F82" s="6" t="n"/>
@@ -4524,12 +4524,12 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>MABOROSHI</t>
+          <t>KIRIBARI</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>部屋が暗くなり映った人が床から投影されたホログラムになる。走査線と輪郭の光で透けて立ち速く動いたところから信号が裂けて横にずれ少し前の自分の残像が遅れてついてくる。はじめは普通のカメラでボタンを押すと暗転して像が床から一行ずつ組み上がる。撮影と録画ができる。</t>
+          <t>カメラの画面が何十枚もの写真を壁に貼り合わせたコラージュになる。写真は一枚ずつ別の瞬間に撮り直されるので止まれば一枚の絵に揃い動くとあなたの体がばらばらの時刻に割れて写真が揺れる。はじめは普通のカメラでボタンを押すとシャッターが光って映像が写真の束に割れる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F83" s="6" t="n"/>
@@ -4555,12 +4555,12 @@
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>ZUKEI</t>
+          <t>MABOROSHI</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+          <t>部屋が暗くなり映った人が床から投影されたホログラムになる。走査線と輪郭の光で透けて立ち速く動いたところから信号が裂けて横にずれ少し前の自分の残像が遅れてついてくる。はじめは普通のカメラでボタンを押すと暗転して像が床から一行ずつ組み上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F84" s="6" t="n"/>
@@ -4570,10 +4570,41 @@
         </is>
       </c>
     </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>ZUKEI</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="n"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G84"/>
+  <autoFilter ref="A1:G85"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4661,6 +4692,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4807,7 +4839,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$84,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$85,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4830,7 +4862,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$84,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$85,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4853,7 +4885,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$84,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$85,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4874,7 +4906,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TANZAKU: portrait printed on hanging ribbons that twist to gold where you move
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017KRmMT7pQsv484VXvsupf9
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4601,10 +4601,41 @@
         </is>
       </c>
     </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>TANZAKU</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>映った人が天井から吊られた何十本もの細い短冊に刷られたモノクロの肖像になる。動いたところの短冊だけがねじれて翻り裏の金箔がひらめき止まれば一枚の肖像に戻る。はじめは普通のカメラでボタンを押すと短冊が端から一回転して肖像に切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="n"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G85"/>
+  <autoFilter ref="A1:G86"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4693,6 +4724,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4839,7 +4871,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$85,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$86,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4862,7 +4894,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$85,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$86,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4885,7 +4917,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$85,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$86,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4906,7 +4938,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
RYUSEN: wind-tunnel smoke streamlines that part around your body
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017KRmMT7pQsv484VXvsupf9
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4617,12 +4617,12 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>TANZAKU</t>
+          <t>RYUSEN</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>映った人が天井から吊られた何十本もの細い短冊に刷られたモノクロの肖像になる。動いたところの短冊だけがねじれて翻り裏の金箔がひらめき止まれば一枚の肖像に戻る。はじめは普通のカメラでボタンを押すと短冊が端から一回転して肖像に切り替わる。撮影と録画ができる。</t>
+          <t>暗い風洞の中に立つと白い煙の流線があなたの体の形に沿って分かれ頭や肩をなめて流れていく。止まれば静かな層流で動けば体のうしろに渦が巻いて線がちぎれ一本だけ赤い染料の線が混じる。はじめは普通のカメラでボタンを押すと暗転して煙の前線が押し寄せる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F86" s="6" t="n"/>
@@ -4632,10 +4632,41 @@
         </is>
       </c>
     </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>TANZAKU</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>映った人が天井から吊られた何十本もの細い短冊に刷られたモノクロの肖像になる。動いたところの短冊だけがねじれて翻り裏の金箔がひらめき止まれば一枚の肖像に戻る。はじめは普通のカメラでボタンを押すと短冊が端から一回転して肖像に切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="n"/>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G86"/>
+  <autoFilter ref="A1:G87"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4725,6 +4756,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4871,7 +4903,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$86,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$87,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4894,7 +4926,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$86,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$87,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4917,7 +4949,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$86,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$87,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4938,7 +4970,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
ITOKAKE: a live string-art portrait whose threads snap where you move
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017KRmMT7pQsv484VXvsupf9
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4617,12 +4617,12 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>RYUSEN</t>
+          <t>ITOKAKE</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>暗い風洞の中に立つと白い煙の流線があなたの体の形に沿って分かれ頭や肩をなめて流れていく。止まれば静かな層流で動けば体のうしろに渦が巻いて線がちぎれ一本だけ赤い染料の線が混じる。はじめは普通のカメラでボタンを押すと暗転して煙の前線が押し寄せる。撮影と録画ができる。</t>
+          <t>映った人が円く打った二百本の釘のあいだに何千本もの白い糸を張った糸かけの肖像になる。動いたところを通る糸は金色に弾けて弦の音で鳴り止まれば一本ずつ張り直されて顔に戻る。はじめは普通のカメラでボタンを押すと何も無い板に糸が高速で張られて肖像が編み上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F86" s="6" t="n"/>
@@ -4648,12 +4648,12 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>TANZAKU</t>
+          <t>RYUSEN</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>映った人が天井から吊られた何十本もの細い短冊に刷られたモノクロの肖像になる。動いたところの短冊だけがねじれて翻り裏の金箔がひらめき止まれば一枚の肖像に戻る。はじめは普通のカメラでボタンを押すと短冊が端から一回転して肖像に切り替わる。撮影と録画ができる。</t>
+          <t>暗い風洞の中に立つと白い煙の流線があなたの体の形に沿って分かれ頭や肩をなめて流れていく。止まれば静かな層流で動けば体のうしろに渦が巻いて線がちぎれ一本だけ赤い染料の線が混じる。はじめは普通のカメラでボタンを押すと暗転して煙の前線が押し寄せる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F87" s="6" t="n"/>
@@ -4663,10 +4663,41 @@
         </is>
       </c>
     </row>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>TANZAKU</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>映った人が天井から吊られた何十本もの細い短冊に刷られたモノクロの肖像になる。動いたところの短冊だけがねじれて翻り裏の金箔がひらめき止まれば一枚の肖像に戻る。はじめは普通のカメラでボタンを押すと短冊が端から一回転して肖像に切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="n"/>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G87"/>
+  <autoFilter ref="A1:G88"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4757,6 +4788,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4903,7 +4935,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$87,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$88,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4926,7 +4958,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$87,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$88,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4949,7 +4981,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$87,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$88,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -4970,7 +5002,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
UTSUWA: the person as a glass vessel of whisky that sloshes as they move
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017KRmMT7pQsv484VXvsupf9
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4694,10 +4694,41 @@
         </is>
       </c>
     </row>
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>UTSUWA</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>映った人が琥珀色の酒を満たしたガラスの器になる。顔は透きとおったガラスに体は光を通す琥珀になり体を横に動かすと中の酒が大きく揺れて跳べば飛沫が上がりタップすると氷がひとつ浮かぶ。はじめは普通のカメラでボタンを押すと頭の上から酒が注がれて体の底から満ちていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="n"/>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G88"/>
+  <autoFilter ref="A1:G89"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4789,6 +4820,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4935,7 +4967,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$88,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$89,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4958,7 +4990,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$88,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$89,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4981,7 +5013,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$88,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$89,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5002,7 +5034,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
SEKIGAI: the person as a thermal image; motion flares red, residual heat lingers and rises
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sc5zVvG6mry6N25LT2aXXp
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4725,10 +4725,41 @@
         </is>
       </c>
     </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>SEKIGAI</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>映った人が赤外線カメラの熱の像になり顔と手が白く灼ける。動いたところは赤く発熱して体の形の残熱が壁に残ったまま冷えて立ちのぼる。はじめは普通のカメラでボタンを押すとシャッター音とともに校正画面が入り冷えた像から体温が浮かび上がる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="n"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G89"/>
+  <autoFilter ref="A1:G90"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4821,6 +4852,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4967,7 +4999,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$89,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$90,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4990,7 +5022,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$89,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$90,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5013,7 +5045,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$89,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$90,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5034,7 +5066,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KAIROU: a feedback corridor of your past selves sinking into Klein blue
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sc5zVvG6mry6N25LT2aXXp
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4741,12 +4741,12 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>SEKIGAI</t>
+          <t>KAIROU</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>映った人が赤外線カメラの熱の像になり顔と手が白く灼ける。動いたところは赤く発熱して体の形の残熱が壁に残ったまま冷えて立ちのぼる。はじめは普通のカメラでボタンを押すとシャッター音とともに校正画面が入り冷えた像から体温が浮かび上がる。撮影と録画ができる。</t>
+          <t>映った人のうしろに少し前の自分が一人ずつ縮みながら奥の消失点へ並び深い青に沈んでいく。止まれば静かなトンネルで横に動けば遅れた自分たちの列がうねって回廊ごとねじれる。はじめは普通のカメラでボタンを押すと部屋ごとの画面が一枚の額になって奥へ吸い込まれる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F90" s="6" t="n"/>
@@ -4756,10 +4756,41 @@
         </is>
       </c>
     </row>
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>SEKIGAI</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>映った人が赤外線カメラの熱の像になり顔と手が白く灼ける。動いたところは赤く発熱して体の形の残熱が壁に残ったまま冷えて立ちのぼる。はじめは普通のカメラでボタンを押すとシャッター音とともに校正画面が入り冷えた像から体温が浮かび上がる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="n"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G90"/>
+  <autoFilter ref="A1:G91"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4853,6 +4884,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4999,7 +5031,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$90,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$91,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5022,7 +5054,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$90,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$91,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5045,7 +5077,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$90,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$91,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5066,7 +5098,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
Remove HAMON and HARUKA at the owner's request
Both read as weak: HARUKA was essentially a virtual background and HAMON
changed only the space around the person, not the person. Cards, works.csv
rows, register entries and xlsx rows removed; replacements follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4462,12 +4462,12 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>HAMON</t>
+          <t>KIRIBARI</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>映った人の輪郭からその瞬間の自分の形をした線が波紋のように広がっていく。止まっていればゆっくり一本ずつ動けばゆがんだ輪がいくつも重なってあふれ出し動いた瞬間の輪だけが差し色になる。はじめは普通のカメラでボタンを押すと暗転して体から三重の輪が放たれる。撮影と録画ができる。</t>
+          <t>カメラの画面が何十枚もの写真を壁に貼り合わせたコラージュになる。写真は一枚ずつ別の瞬間に撮り直されるので止まれば一枚の絵に揃い動くとあなたの体がばらばらの時刻に割れて写真が揺れる。はじめは普通のカメラでボタンを押すとシャッターが光って映像が写真の束に割れる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F81" s="6" t="n"/>
@@ -4493,12 +4493,12 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>HARUKA</t>
+          <t>MABOROSHI</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>部屋が消えて映った人だけが映画のポスターのような遠い景色の前に立つ。大きな月と山並み・夕暮れの砂丘・霧の森。頭を動かすと景色が奥行きのとおりにずれて窓の向こうに本当に世界があるように見える。はじめは普通のカメラでボタンを押すと景色が下から順にせり上がる。撮影と録画ができる。</t>
+          <t>部屋が暗くなり映った人が床から投影されたホログラムになる。走査線と輪郭の光で透けて立ち速く動いたところから信号が裂けて横にずれ少し前の自分の残像が遅れてついてくる。はじめは普通のカメラでボタンを押すと暗転して像が床から一行ずつ組み上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F82" s="6" t="n"/>
@@ -4524,12 +4524,12 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>KIRIBARI</t>
+          <t>ZUKEI</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>カメラの画面が何十枚もの写真を壁に貼り合わせたコラージュになる。写真は一枚ずつ別の瞬間に撮り直されるので止まれば一枚の絵に揃い動くとあなたの体がばらばらの時刻に割れて写真が揺れる。はじめは普通のカメラでボタンを押すとシャッターが光って映像が写真の束に割れる。撮影と録画ができる。</t>
+          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F83" s="6" t="n"/>
@@ -4550,17 +4550,17 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>MABOROSHI</t>
+          <t>ITOKAKE</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>部屋が暗くなり映った人が床から投影されたホログラムになる。走査線と輪郭の光で透けて立ち速く動いたところから信号が裂けて横にずれ少し前の自分の残像が遅れてついてくる。はじめは普通のカメラでボタンを押すと暗転して像が床から一行ずつ組み上がる。撮影と録画ができる。</t>
+          <t>映った人が円く打った二百本の釘のあいだに何千本もの白い糸を張った糸かけの肖像になる。動いたところを通る糸は金色に弾けて弦の音で鳴り止まれば一本ずつ張り直されて顔に戻る。はじめは普通のカメラでボタンを押すと何も無い板に糸が高速で張られて肖像が編み上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F84" s="6" t="n"/>
@@ -4581,17 +4581,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>ZUKEI</t>
+          <t>RYUSEN</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>映った人がバウハウスのポスターのような図形の肖像になる。四分円・半円・正方形の墨と朱で組まれ動いたところの図形はくるりと回って朱に弾け止まればまた顔に組み直る。はじめは普通のカメラでボタンを押すと紙の升目が映像を覆って図形が刷られていく。撮影と録画ができる。</t>
+          <t>暗い風洞の中に立つと白い煙の流線があなたの体の形に沿って分かれ頭や肩をなめて流れていく。止まれば静かな層流で動けば体のうしろに渦が巻いて線がちぎれ一本だけ赤い染料の線が混じる。はじめは普通のカメラでボタンを押すと暗転して煙の前線が押し寄せる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F85" s="6" t="n"/>
@@ -4617,12 +4617,12 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>ITOKAKE</t>
+          <t>TANZAKU</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>映った人が円く打った二百本の釘のあいだに何千本もの白い糸を張った糸かけの肖像になる。動いたところを通る糸は金色に弾けて弦の音で鳴り止まれば一本ずつ張り直されて顔に戻る。はじめは普通のカメラでボタンを押すと何も無い板に糸が高速で張られて肖像が編み上がる。撮影と録画ができる。</t>
+          <t>映った人が天井から吊られた何十本もの細い短冊に刷られたモノクロの肖像になる。動いたところの短冊だけがねじれて翻り裏の金箔がひらめき止まれば一枚の肖像に戻る。はじめは普通のカメラでボタンを押すと短冊が端から一回転して肖像に切り替わる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F86" s="6" t="n"/>
@@ -4648,12 +4648,12 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>RYUSEN</t>
+          <t>UTSUWA</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>暗い風洞の中に立つと白い煙の流線があなたの体の形に沿って分かれ頭や肩をなめて流れていく。止まれば静かな層流で動けば体のうしろに渦が巻いて線がちぎれ一本だけ赤い染料の線が混じる。はじめは普通のカメラでボタンを押すと暗転して煙の前線が押し寄せる。撮影と録画ができる。</t>
+          <t>映った人が琥珀色の酒を満たしたガラスの器になる。顔は透きとおったガラスに体は光を通す琥珀になり体を横に動かすと中の酒が大きく揺れて跳べば飛沫が上がりタップすると氷がひとつ浮かぶ。はじめは普通のカメラでボタンを押すと頭の上から酒が注がれて体の底から満ちていく。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F87" s="6" t="n"/>
@@ -4674,17 +4674,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>TANZAKU</t>
+          <t>KAIROU</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>映った人が天井から吊られた何十本もの細い短冊に刷られたモノクロの肖像になる。動いたところの短冊だけがねじれて翻り裏の金箔がひらめき止まれば一枚の肖像に戻る。はじめは普通のカメラでボタンを押すと短冊が端から一回転して肖像に切り替わる。撮影と録画ができる。</t>
+          <t>映った人のうしろに少し前の自分が一人ずつ縮みながら奥の消失点へ並び深い青に沈んでいく。止まれば静かなトンネルで横に動けば遅れた自分たちの列がうねって回廊ごとねじれる。はじめは普通のカメラでボタンを押すと部屋ごとの画面が一枚の額になって奥へ吸い込まれる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F88" s="6" t="n"/>
@@ -4705,17 +4705,17 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>UTSUWA</t>
+          <t>SEKIGAI</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>映った人が琥珀色の酒を満たしたガラスの器になる。顔は透きとおったガラスに体は光を通す琥珀になり体を横に動かすと中の酒が大きく揺れて跳べば飛沫が上がりタップすると氷がひとつ浮かぶ。はじめは普通のカメラでボタンを押すと頭の上から酒が注がれて体の底から満ちていく。撮影と録画ができる。</t>
+          <t>映った人が赤外線カメラの熱の像になり顔と手が白く灼ける。動いたところは赤く発熱して体の形の残熱が壁に残ったまま冷えて立ちのぼる。はじめは普通のカメラでボタンを押すとシャッター音とともに校正画面が入り冷えた像から体温が浮かび上がる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F89" s="6" t="n"/>
@@ -4725,72 +4725,10 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="30" customHeight="1">
-      <c r="A90" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="3" t="inlineStr">
-        <is>
-          <t>〇</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>KAIROU</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>映った人のうしろに少し前の自分が一人ずつ縮みながら奥の消失点へ並び深い青に沈んでいく。止まれば静かなトンネルで横に動けば遅れた自分たちの列がうねって回廊ごとねじれる。はじめは普通のカメラでボタンを押すと部屋ごとの画面が一枚の額になって奥へ吸い込まれる。撮影と録画ができる。</t>
-        </is>
-      </c>
-      <c r="F90" s="6" t="n"/>
-      <c r="G90" s="2" t="inlineStr">
-        <is>
-          <t>エフェクト</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="30" customHeight="1">
-      <c r="A91" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>〇</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>SEKIGAI</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="inlineStr">
-        <is>
-          <t>映った人が赤外線カメラの熱の像になり顔と手が白く灼ける。動いたところは赤く発熱して体の形の残熱が壁に残ったまま冷えて立ちのぼる。はじめは普通のカメラでボタンを押すとシャッター音とともに校正画面が入り冷えた像から体温が浮かび上がる。撮影と録画ができる。</t>
-        </is>
-      </c>
-      <c r="F91" s="6" t="n"/>
-      <c r="G91" s="2" t="inlineStr">
-        <is>
-          <t>エフェクト</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G91"/>
+  <autoFilter ref="A1:G89"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4883,8 +4821,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5031,7 +4967,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$91,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$89,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5054,7 +4990,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$91,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$89,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5077,7 +5013,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$91,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$89,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5098,7 +5034,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TAISHO: the frame folded along the face's own midline into a symmetric face
A line is fitted through 22 FaceLandmarker midline points (principal axis,
aspect-corrected screen pixels) and every pixel past it is replaced by its
mirror image, so tilting or turning the head reshapes the face. Tap swaps
the kept half. Checked against real webcam footage with the real model.
Starts as the plain camera. Card, works.csv, register and xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4725,10 +4725,41 @@
         </is>
       </c>
     </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>TAISHO</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>顔のまんなかの線で画面が折り返されあなたは完全に左右対称の顔になる。折り目は鼻筋についてくるので首をかしげたり横を向いたりすると顔が別人に化けタップで右の顔と左の顔が入れ替わる。はじめは普通のカメラでボタンを押すと額から顎へ画面が折り返されていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="n"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G89"/>
+  <autoFilter ref="A1:G90"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4821,6 +4852,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4967,7 +4999,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$89,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$90,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -4990,7 +5022,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$89,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$90,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5013,7 +5045,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$89,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$90,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5034,7 +5066,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KAGEBOSHI: a lamp-lit room where your shadow on the wall lags a second behind
Person masks are kept with timestamps in a 64-layer texture array; the
layer nearest (now - delay) is projected from a side lamp onto the wall as
a hard shadow, never over the person. Tap leaves the shadow on the wall in
its pose; tap again calls it back. Checked against real webcam footage
with the real segmenter. Starts as the plain camera. Card, works.csv,
register and xlsx updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4741,12 +4741,12 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>TAISHO</t>
+          <t>KAGEBOSHI</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>顔のまんなかの線で画面が折り返されあなたは完全に左右対称の顔になる。折り目は鼻筋についてくるので首をかしげたり横を向いたりすると顔が別人に化けタップで右の顔と左の顔が入れ替わる。はじめは普通のカメラでボタンを押すと額から顎へ画面が折り返されていく。撮影と録画ができる。</t>
+          <t>部屋の明かりが落ち横から一灯だけの光があなたを照らして壁に大きな影が落ちる。その影は一秒ほど遅れてあなたを追いかけタップすると影をその姿勢のまま壁に置いていける。はじめは普通のカメラでボタンを押すと暗転して電球が点き壁に影が浮かぶ。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F90" s="6" t="n"/>
@@ -4756,10 +4756,41 @@
         </is>
       </c>
     </row>
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>TAISHO</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>顔のまんなかの線で画面が折り返されあなたは完全に左右対称の顔になる。折り目は鼻筋についてくるので首をかしげたり横を向いたりすると顔が別人に化けタップで右の顔と左の顔が入れ替わる。はじめは普通のカメラでボタンを押すと額から顎へ画面が折り返されていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="n"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G90"/>
+  <autoFilter ref="A1:G91"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4853,6 +4884,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4999,7 +5031,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$90,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$91,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5022,7 +5054,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$90,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$91,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5045,7 +5077,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$90,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$91,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5066,7 +5098,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
Register CUBRICK TRIANGLE STAR in the gallery, works.csv, xlsx and register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qqwbi4o5nHTavi6kGESB1F
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4787,10 +4787,41 @@
         </is>
       </c>
     </row>
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>キューブリック・トライアングル・スター</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>人差し指・中指・薬指を立てるとその指がさす先に箱が一個ずつ浮かび指を閉じるかもう片方の手の同じ指に当てると箱が移る。形は箱・球・スター・三角から選べて色や大きさ・白黒フラッシュ・オーラも切り替えられる。</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="n"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G91"/>
+  <autoFilter ref="A1:G92"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4885,6 +4916,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5031,7 +5063,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$91,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$92,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5054,7 +5086,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$91,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$92,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5077,7 +5109,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$91,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$92,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5098,7 +5130,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
Add HAMON: ripples spread from your outline, engraved-line portrait
The person becomes a fine-line engraving and their outline keeps emitting
concentric ripples; moving bunches the waves ahead and leaves a vermilion
wake behind. Starts on the plain camera; the switch opens one ring from the
body. Card, works.csv, xlsx and register updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VKSzYqDB4jEUzPqgwe7mxY
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4818,10 +4818,41 @@
         </is>
       </c>
     </row>
+    <row r="93" ht="30" customHeight="1">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>HAMON</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>映った人が細い線で彫られた版画になり体の輪郭から波紋が絶えず広がる。止まれば静かな同心円で歩けば波が前に詰まって後ろに航跡が伸び速く動いた瞬間の輪だけが朱に染まる。はじめは普通のカメラでボタンを押すと体から輪が開いて画面が線の世界に塗り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="n"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G92"/>
+  <autoFilter ref="A1:G93"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4917,6 +4948,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5063,7 +5095,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$92,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$93,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5086,7 +5118,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$92,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$93,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5109,7 +5141,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$92,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$93,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5130,7 +5162,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
Add KONTENGI: a brass armillary sphere around your head
The person becomes a warm-black monochrome portrait and five brass rings
orbit the head, their back arcs hidden behind the body. Head turns and
body motion torque the gimbals in alternating directions; spin opens the
sphere and leaves gold trails. Starts on the plain camera; the switch
sinks the room and flies the rings in. Card, works.csv, xlsx and register
updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VKSzYqDB4jEUzPqgwe7mxY
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4849,10 +4849,41 @@
         </is>
       </c>
     </row>
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>KONTENGI</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>映った人が暗い温黒調の肖像写真になり頭のまわりに真鍮の渾天儀が組み上がる。首を振ったり歩いたりすると環がジャイロのように互い違いに回りだし速いほど大きく開いて金の残光を引く。はじめは普通のカメラでボタンを押すと部屋が沈んで環が回りながら飛んでくる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F94" s="6" t="n"/>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G93"/>
+  <autoFilter ref="A1:G94"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4949,6 +4980,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5095,7 +5127,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$93,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$94,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5118,7 +5150,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$93,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$94,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5141,7 +5173,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$93,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$94,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5162,7 +5194,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
Add OMOCHABAKO: wave to flip into a pop collage with a glitch silhouette
A reproduction of the screen recording the owner shared: an open-hand wave
sweeps the camera into a dense pop collage (candy tubes, ribbons, skulls,
hiragana tiles) that cuts every second, with the person as a datamosh
mosaic silhouette. A 大人 style swaps it for a monochrome-and-vermilion
collage with slower cuts and grain. Card, works.csv, xlsx and register
updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VKSzYqDB4jEUzPqgwe7mxY
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4880,10 +4880,41 @@
         </is>
       </c>
     </row>
+    <row r="95" ht="30" customHeight="1">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>OMOCHABAKO</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが見せてくれた動画の再現。手を開いて左右に振るとカメラが左からピクセルのブロックに崩れて映った人はグリッチのモザイクで埋まったシルエットになりまわりがキャンディ柄の管・三角・ドクロ・ひらがなのタイルでぎっしり埋まる。場面は一秒ごとに切り替わり「大人」に切り替えるとモノクロと朱一色の静かなコラージュになる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="n"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G94"/>
+  <autoFilter ref="A1:G95"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4981,6 +5012,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5127,7 +5159,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$94,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$95,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5150,7 +5182,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$94,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$95,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5173,7 +5205,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$94,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$95,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5194,7 +5226,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
RENSHA, ZANZOU: start on the plain camera and add a 🎲 random button
Both now open on the plain camera and switch into the effect with a
button (RENSHA: the room drops to dark and one strobe fires; ZANZOU: the
drawing sweeps down behind a hatched band), and back again. 🎲 re-rolls
the look: RENSHA the clone colour pair, rate, life and glow; ZANZOU the
three trail colours, delay, line density, contrast and hatch angle.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VKSzYqDB4jEUzPqgwe7mxY
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -3878,7 +3878,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>動くとそのぶん自分の姿がストロボの分身として空中に焼き付いていくエフェクト。速く動くほど分身は詰まって並び止まればいまの自分だけが残る。撮影と録画ができる。</t>
+          <t>動くとそのぶん自分の姿がストロボの分身として空中に焼き付いていくエフェクト。速く動くほど分身は詰まって並び止まればいまの自分だけが残る。撮影と録画ができる。はじめは普通のカメラでボタンを押すとストロボが光って切り替わり🎲で分身の色と連写がランダムに変わる。</t>
         </is>
       </c>
       <c r="F62" s="6" t="n"/>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>カメラに映った人物だけを白黒のクロスハッチ線画にするエフェクト。動いた跡は青・マゼンタ・黄の色つきシルエットになって遅れてついてくる。線の細かさ・遅れ・コントラスト・配色を操作パネルで調整できる。</t>
+          <t>カメラに映った人物だけを白黒のクロスハッチ線画にするエフェクト。動いた跡は青・マゼンタ・黄の色つきシルエットになって遅れてついてくる。線の細かさ・遅れ・コントラスト・配色を操作パネルで調整できる。はじめは普通のカメラでボタンを押すと線画が上から塗り替わり🎲で残像の色と線がランダムに変わる。</t>
         </is>
       </c>
       <c r="F64" s="6" t="n"/>

</xml_diff>

<commit_message>
SABUN: motion-only relief on a wall, with a burn-in ghost
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr9qRGo5QDuSaEwjybXfL9
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5082,12 +5082,12 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>SHINGOU</t>
+          <t>IREZUMI</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>白い壁の前であなたのシルエットが黒く抜かれその中をバーコード・点滅する格子・波形・1ビットの顔が帯になって流れる。止まれば整然と流れ動けば体が横の帯ごとに裂けてずれ帯の中身が切り替わる。はじめは普通のカメラでボタンを押すと上から帯ごとに入れ替わる。撮影と録画ができる。</t>
+          <t>赤い地の前で映った人が白黒の肖像になり顔から首まで黒い紋様の入れ墨が入る。波線・稲妻・渦・菱の紋様は顔に貼りついて首の動きについてくる。目と唇は素肌のまま。動くと線が流れ入れたての墨が赤く滲む。タップで図案が彫り直され撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F101" s="6" t="n"/>
@@ -5097,10 +5097,165 @@
         </is>
       </c>
     </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>MUKU</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>映った人が白い紙にシルクスクリーンで刷られたポップアートの一枚になる。体は黄色のベタに黒いインクの斑と太い輪郭線。指でなぞると刷りがステッカーのようにめくれて下から桃色のあなたが出てくる。動くと黄色の版がずれてついてくる。タップで色版が替わり撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="n"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>MYAKUDO</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>カメラに映るものすべてが黒地に何十本も重なる白い波形になる。明るいところほど線が持ち上がり手前の線が奥の線を隠すので地下鉄の車内も部屋も山脈のような信号の図になる。動いたところは線が電波のように震えタップで色が替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F103" s="6" t="n"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="30" customHeight="1">
+      <c r="A104" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>SHINGOU</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>白い壁の前であなたのシルエットが黒く抜かれその中をバーコード・点滅する格子・波形・1ビットの顔が帯になって流れる。止まれば整然と流れ動けば体が横の帯ごとに裂けてずれ帯の中身が切り替わる。はじめは普通のカメラでボタンを押すと上から帯ごとに入れ替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F104" s="6" t="n"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>SUISOU</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>線だけの立方体（球にも切り替えられる）が宙に浮かび中に青い水が入っている。両手で持つとあいだに来て離すほど大きく両手を回すと一緒に回り放すとくるくる回り続ける。持っていないときはゆっくり浮かぶ。中の水は千数百粒の本物の粒子流体。大きさと色と水の量を変えられ撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F105" s="6" t="n"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>SABUN</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>画面が灰色の壁になり止まっているものはすべて消える。動いたときだけあなたが白と黒の浮彫になって現れ朱の残像が後を追う。タップで部屋を焼き付けると自分の抜け殻と並べる。はじめは普通のカメラでボタンを押すと朱の線が壁を引き下ろす。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="n"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G101"/>
+  <autoFilter ref="A1:G106"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5205,6 +5360,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId105"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5351,7 +5511,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$101,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$106,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5374,7 +5534,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$101,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$106,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5397,7 +5557,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$101,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$106,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5418,7 +5578,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
MEMAI: your outline as a vortex of concentric rings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr9qRGo5QDuSaEwjybXfL9
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G106"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5237,12 +5237,12 @@
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>SABUN</t>
+          <t>MEMAI</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>画面が灰色の壁になり止まっているものはすべて消える。動いたときだけあなたが白と黒の浮彫になって現れ朱の残像が後を追う。タップで部屋を焼き付けると自分の抜け殻と並べる。はじめは普通のカメラでボタンを押すと朱の線が壁を引き下ろす。撮影と録画ができる。</t>
+          <t>あなたの輪郭が象牙・深紅・墨の帯になって何重にも外へ広がり続ける渦のポスター。帯は少し前のあなたの形なので動くほど渦がよじれて開き止まれば静かな同心の輪に戻る。タップで回転が逆向きに。はじめは普通のカメラでボタンを押すと部屋が沈んで体から輪が開く。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F106" s="6" t="n"/>
@@ -5252,10 +5252,41 @@
         </is>
       </c>
     </row>
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>SABUN</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>画面が灰色の壁になり止まっているものはすべて消える。動いたときだけあなたが白と黒の浮彫になって現れ朱の残像が後を追う。タップで部屋を焼き付けると自分の抜け殻と並べる。はじめは普通のカメラでボタンを押すと朱の線が壁を引き下ろす。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="n"/>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G106"/>
+  <autoFilter ref="A1:G107"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5365,6 +5396,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5511,7 +5543,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$106,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$107,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5534,7 +5566,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$106,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$107,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5557,7 +5589,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$106,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$107,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5578,7 +5610,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TSUBASA: black wings unfold from your shoulders
A monochrome portrait on studio paper; wings rigged to the pose open
with your arms and beat once when you jump, shedding feathers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXWzfYcpzbGCS8BVmeBRKc
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5283,10 +5283,41 @@
         </is>
       </c>
     </row>
+    <row r="108" ht="30" customHeight="1">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>TSUBASA</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>灰色のスタジオ紙の前で映った人がモノクロの肖像になり肩から大きな黒い翼がひらく。腕を広げれば翼も広がり跳べば一度羽ばたいて羽根が舞い散る。はじめは普通のカメラでボタンを押すと暗転して翼がほどける。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="n"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G107"/>
+  <autoFilter ref="A1:G108"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5397,6 +5428,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5543,7 +5575,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$107,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$108,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5566,7 +5598,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$107,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$108,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5589,7 +5621,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$107,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$108,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5610,7 +5642,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
SENKOU: anamorphic flares from your eyes
A cinemascope night grade; blue lens flares lock to your irises, leave
trails when you turn your head, and ignite across the frame when you
close your eyes and open them again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXWzfYcpzbGCS8BVmeBRKc
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>TSUBASA</t>
+          <t>SENKOU</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>灰色のスタジオ紙の前で映った人がモノクロの肖像になり肩から大きな黒い翼がひらく。腕を広げれば翼も広がり跳べば一度羽ばたいて羽根が舞い散る。はじめは普通のカメラでボタンを押すと暗転して翼がほどける。撮影と録画ができる。</t>
+          <t>画面がシネスコの夜の映画になりあなたの瞳から青いアナモルフィックの光芒が横一文字に走る。首を振ると光の軌跡が残り目を閉じてから開くと光が画面の端から端まで閃く。二人で映れば四つの光。はじめは普通のカメラでボタンを押すと暗転して光が入る。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F108" s="6" t="n"/>
@@ -5314,10 +5314,41 @@
         </is>
       </c>
     </row>
+    <row r="109" ht="30" customHeight="1">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>TSUBASA</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>灰色のスタジオ紙の前で映った人がモノクロの肖像になり肩から大きな黒い翼がひらく。腕を広げれば翼も広がり跳べば一度羽ばたいて羽根が舞い散る。はじめは普通のカメラでボタンを押すと暗転して翼がほどける。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="n"/>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G108"/>
+  <autoFilter ref="A1:G109"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5429,6 +5460,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5575,7 +5607,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$108,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$109,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5598,7 +5630,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$108,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$109,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5621,7 +5653,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$108,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$109,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5642,7 +5674,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KATADORI: your face as a living plaster cast
The live 3D face mesh becomes a plaster, chrome or bronze mask in a dark
gallery. Moving leaves casts along the path, fast moves shatter them onto
the floor, and a tap keeps an expression. CLAUDE.md: one elaborate piece
per night from now on.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXWzfYcpzbGCS8BVmeBRKc
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>SENKOU</t>
+          <t>KATADORI</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>画面がシネスコの夜の映画になりあなたの瞳から青いアナモルフィックの光芒が横一文字に走る。首を振ると光の軌跡が残り目を閉じてから開くと光が画面の端から端まで閃く。二人で映れば四つの光。はじめは普通のカメラでボタンを押すと暗転して光が入る。撮影と録画ができる。</t>
+          <t>顔が生きている彫刻になる。暗いギャラリーに自分の顔を型取りした石膏の面が浮かびゆっくり回って横顔まで見せる。首を動かせば軌跡に型が並んで連続写真のような彫刻になり速く振れば砕けて床に崩れ落ちる。タップでその表情の型を残して群像を組める。石膏・クロム・青銅。はじめは普通のカメラでボタンを押すと走査線が顔をなぞって石膏になる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F108" s="6" t="n"/>
@@ -5330,12 +5330,12 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>TSUBASA</t>
+          <t>SENKOU</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>灰色のスタジオ紙の前で映った人がモノクロの肖像になり肩から大きな黒い翼がひらく。腕を広げれば翼も広がり跳べば一度羽ばたいて羽根が舞い散る。はじめは普通のカメラでボタンを押すと暗転して翼がほどける。撮影と録画ができる。</t>
+          <t>画面がシネスコの夜の映画になりあなたの瞳から青いアナモルフィックの光芒が横一文字に走る。首を振ると光の軌跡が残り目を閉じてから開くと光が画面の端から端まで閃く。二人で映れば四つの光。はじめは普通のカメラでボタンを押すと暗転して光が入る。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F109" s="6" t="n"/>
@@ -5345,10 +5345,41 @@
         </is>
       </c>
     </row>
+    <row r="110" ht="30" customHeight="1">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>TSUBASA</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>灰色のスタジオ紙の前で映った人がモノクロの肖像になり肩から大きな黒い翼がひらく。腕を広げれば翼も広がり跳べば一度羽ばたいて羽根が舞い散る。はじめは普通のカメラでボタンを押すと暗転して翼がほどける。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="n"/>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G109"/>
+  <autoFilter ref="A1:G110"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5461,6 +5492,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId109"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5607,7 +5639,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$109,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$110,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5630,7 +5662,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$109,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$110,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5653,7 +5685,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$109,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$110,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5674,7 +5706,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TOUSHI: your body as a moving radiograph
The skeleton, lungs and organs are rebuilt every frame from the pose and
hand landmarks as ~1300 analytic primitives per person (hollow tubes,
ellipsoidal shells, rounded boxes, fan-shaped plates; curved bones are
mitred chains that brighten where they run along the ray) and exposed
through Beer-Lambert attenuation. Dark lung fields with vessels, a beating
heart shadow and bowel gas; heart and breathing rates rise with motion.
Fast motion fires an X-ray strobe that leaves ghost exposures on the film.
FILM, FLUORO and an 1895 glass plate.

Also: gallery card, works.csv row, xlsx, register entry, and a note in
CLAUDE.md on what made this an elaborate piece.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXWzfYcpzbGCS8BVmeBRKc
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5361,12 +5361,12 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>TSUBASA</t>
+          <t>TOUSHI</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>灰色のスタジオ紙の前で映った人がモノクロの肖像になり肩から大きな黒い翼がひらく。腕を広げれば翼も広がり跳べば一度羽ばたいて羽根が舞い散る。はじめは普通のカメラでボタンを押すと暗転して翼がほどける。撮影と録画ができる。</t>
+          <t>体が動くレントゲン写真になる。頭蓋骨・肋骨・骨盤・手の小さな骨まで X 線の写り方で透け黒い肺野の中で心臓の影が打つ。動くほど心拍と呼吸が上がる。速く動くと X 線が連写され骨の残像が多重露光で焼き付く。FILM・FLUORO・1895 年のガラス乾板（薬指に指輪）。はじめは普通のカメラでボタンを押すとコリメータの光が当たり露光される。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F110" s="6" t="n"/>
@@ -5376,10 +5376,41 @@
         </is>
       </c>
     </row>
+    <row r="111" ht="30" customHeight="1">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>TSUBASA</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>灰色のスタジオ紙の前で映った人がモノクロの肖像になり肩から大きな黒い翼がひらく。腕を広げれば翼も広がり跳べば一度羽ばたいて羽根が舞い散る。はじめは普通のカメラでボタンを押すと暗転して翼がほどける。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="n"/>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G110"/>
+  <autoFilter ref="A1:G111"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5493,6 +5524,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId110"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5639,7 +5671,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$110,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$111,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5662,7 +5694,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$110,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$111,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5685,7 +5717,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$110,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$111,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5706,7 +5738,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KINPAKU: a Klimt golden portrait
Face and hands stay painted skin; the body becomes a gold-leaf mosaic
(ADELE / KUSS / SPIRALE). Moving peels gold flakes off the trailing
edge and leaves a fading gold imprint of the motif on the bronze ground.
Light rakes across the gold with the head. Plain camera <-> gilding switch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xs816qqPJCudaFfEUYSzc
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5407,10 +5407,41 @@
         </is>
       </c>
     </row>
+    <row r="112" ht="30" customHeight="1">
+      <c r="A112" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>KINPAKU</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>クリムトの黄金の肖像画になる。顔と手は白く描かれたまま服と体は目・渦・市松の金箔のモザイクになる。動くと金箔が剥がれて舞いいた場所に金の文様がしばらく残る。タップで ADELE・KUSS・SPIRALE の様式を貼り替える。はじめは普通のカメラでボタンを押すと金箔が一枚ずつ貼られていく。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="n"/>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G111"/>
+  <autoFilter ref="A1:G112"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5525,6 +5556,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId111"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5671,7 +5703,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$111,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$112,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5694,7 +5726,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$111,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$112,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5717,7 +5749,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$111,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$112,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5738,7 +5770,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
NEJIRE: a Francis Bacon portrait that twists with your motion
You become a Bacon study in a flat orange, violet or ochre room inside a
thin white cage. Paint is advected along real optical flow, the face
swirls with the head's turning speed, an open mouth brings down the
pope's vertical curtain, and taps freeze studies into a gilt triptych.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WRBffVfxcCKf51vsaPWvAe
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G112"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5438,10 +5438,41 @@
         </is>
       </c>
     </row>
+    <row r="113" ht="30" customHeight="1">
+      <c r="A113" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>NEJIRE</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>フランシス・ベーコンの肖像画になる。平らな色の部屋と白い檻の中で首を振れば顔がねじれ動いたぶんだけ絵の具が引きずられて跡が残る。口を大きく開けると絵ごと叫びタップで習作を残して三連画に組める。はじめは普通のカメラでボタンを押すと太い刷毛が画面を横切って絵になる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="n"/>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G112"/>
+  <autoFilter ref="A1:G113"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5557,6 +5588,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId112"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5703,7 +5735,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$112,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$113,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5726,7 +5758,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$112,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$113,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5749,7 +5781,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$112,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$113,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5770,7 +5802,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TOKERU: add the owner's melting-scenery piece
The owner's tokeru-keshiki.html, kept as designed (field simulation,
shaders, palette, silence), with the gallery's start screen, gear panel,
camera flip, photo/recording, standard camera error text, landmark
guards and auto-started hand tracking. File upload removed to match the
other pieces.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WRBffVfxcCKf51vsaPWvAe
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5469,10 +5469,41 @@
         </is>
       </c>
     </row>
+    <row r="114" ht="30" customHeight="1">
+      <c r="A114" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>TOKERU</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが持ち込んだ作品（とける景色）。画面を指でなぞるとカメラの景色がガラスのように溶けて渦を巻き虹色の縁を浮かべてから冷えて元に戻る。カメラに手をかざしても溶ける。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="n"/>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G113"/>
+  <autoFilter ref="A1:G114"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5589,6 +5620,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId113"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5735,7 +5767,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$113,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$114,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5758,7 +5790,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$113,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$114,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5781,7 +5813,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$113,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$114,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5802,7 +5834,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
ISSEN: the person redrawn by one oscilloscope beam, and the line plays as stereo X/Y sound
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6W5VkUDTvXTtm68ZcwJaj
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>オーナーが持ち込んだ作品（とける景色）。画面を指でなぞるとカメラの景色がガラスのように溶けて渦を巻き虹色の縁を浮かべてから冷えて元に戻る。カメラに手をかざしても溶ける。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだ作品（とける景色）。画面を指でなぞるとカメラの景色がガラスのように溶けて渦を巻き虹色の縁を浮かべてから冷えて元に戻る。カメラに手をかざしても溶ける。「かたち」でシャボン玉・ドーナツ・スライムがふわふわ浮かび、つかんで投げられる。大きさも調整できる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F114" s="6" t="n"/>
@@ -5500,10 +5500,41 @@
         </is>
       </c>
     </row>
+    <row r="115" ht="30" customHeight="1">
+      <c r="A115" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>ISSEN</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>映った人がオシロスコープの黒い硝子の上で一本の光の線に描き直される。線はそのまま左右の音として鳴り動くと残光が尾を引いて線がばねのように暴れる。タップで姿を焼き付けて重ねられる。はじめは普通のカメラでボタンを押すと像が線から点へ縮みその点がほどけてあなたを描く。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="n"/>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G114"/>
+  <autoFilter ref="A1:G115"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5621,6 +5652,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId114"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5767,7 +5799,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$114,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$115,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5790,7 +5822,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$114,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$115,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5813,7 +5845,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$114,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$115,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5834,7 +5866,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
SEIRETSU: the person pixel-sorted into streaks of light along the way they move
Glitch-art portrait: moving parts are sorted by luminance along their motion
direction and trail off as comet tails; highlights drip when still; a jump or
tap pours the whole body down. Four plates (SILVER, SODIUM, PAPER, COLOR) and a
row-by-row sort sweep between the plain camera and the effect.
Adds the card, works.csv row, xlsx rebuild and register entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjAYv9LVh6abRGkArBYfFq
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5531,10 +5531,41 @@
         </is>
       </c>
     </row>
+    <row r="116" ht="30" customHeight="1">
+      <c r="A116" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>SEIRETSU</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>映った人がピクセルソートのグリッチアートになる。動いたところが動いた向きに明るさ順で並べ替えられ光の筋になって尾を引き止まると明るいところが垂れていく。跳ぶかタップすると体ごと滝のように流れ落ちる。SILVER・SODIUM・PAPER・COLOR の四つの版。はじめは普通のカメラでボタンを押すと画面が一行ずつ並べ替えられて切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F116" s="6" t="n"/>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G115"/>
+  <autoFilter ref="A1:G116"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5653,6 +5684,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5799,7 +5831,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$115,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$116,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5822,7 +5854,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$115,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$116,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5845,7 +5877,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$115,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$116,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5866,7 +5898,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KOGASHI: you, as an old print burning through in the projector gate wherever you move
Warm black-and-white film (grain, 24-frame flicker, gate weave, scratches,
perforated edge) where motion heats the celluloid: it scorches, blisters,
opens a white hole with a glowing amber rim, then cools and closes. A sharp
move slips the frame; a tap ignites. Stocks PRINT, NITRATE, EKTA.
Adds the card, works.csv row, xlsx rebuild and register entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjAYv9LVh6abRGkArBYfFq
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5547,12 +5547,12 @@
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>SEIRETSU</t>
+          <t>KOGASHI</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t>映った人がピクセルソートのグリッチアートになる。動いたところが動いた向きに明るさ順で並べ替えられ光の筋になって尾を引き止まると明るいところが垂れていく。跳ぶかタップすると体ごと滝のように流れ落ちる。SILVER・SODIUM・PAPER・COLOR の四つの版。はじめは普通のカメラでボタンを押すと画面が一行ずつ並べ替えられて切り替わる。撮影と録画ができる。</t>
+          <t>映った人が映写機にかかった温黒調の古いフィルムになる。動いたところからフィルムが焦げて泡立ち琥珀色の縁をつれて白く焼け抜けやがて冷えて閉じる。すばやく動くとコマが滑りタップした場所に火が入る。PRINT・NITRATE・EKTA の三つのフィルム。はじめは普通のカメラでボタンを押すと映写機のランプが瞬いてコマが降りてくる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F116" s="6" t="n"/>
@@ -5562,10 +5562,41 @@
         </is>
       </c>
     </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>SEIRETSU</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>映った人がピクセルソートのグリッチアートになる。動いたところが動いた向きに明るさ順で並べ替えられ光の筋になって尾を引き止まると明るいところが垂れていく。跳ぶかタップすると体ごと滝のように流れ落ちる。SILVER・SODIUM・PAPER・COLOR の四つの版。はじめは普通のカメラでボタンを押すと画面が一行ずつ並べ替えられて切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="n"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G116"/>
+  <autoFilter ref="A1:G117"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5685,6 +5716,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5831,7 +5863,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$116,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$117,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5854,7 +5886,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$116,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$117,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5877,7 +5909,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$116,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$117,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5898,7 +5930,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
MIST TRACKER: add the owner's tracking-ID mist piece to the gallery
Owner-supplied file, mechanism, palette, type and sound kept as designed.
Added the house conventions: start overlay that creates the AudioContext,
⟲ カメラ flip, the standard camera-failure message, snapshot and recording
(with the piece's own audio). Video-file loading and the demo source were
dropped to match the other camera pieces.
Adds the card, works.csv row, xlsx rebuild and register entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjAYv9LVh6abRGkArBYfFq
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5578,12 +5578,12 @@
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>SEIRETSU</t>
+          <t>MIST TRACKER</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t>映った人がピクセルソートのグリッチアートになる。動いたところが動いた向きに明るさ順で並べ替えられ光の筋になって尾を引き止まると明るいところが垂れていく。跳ぶかタップすると体ごと滝のように流れ落ちる。SILVER・SODIUM・PAPER・COLOR の四つの版。はじめは普通のカメラでボタンを押すと画面が一行ずつ並べ替えられて切り替わる。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだ作品。カメラに映った動きに J0925 のような追跡 ID が次々に振られ点どうしが線で結ばれ動いたかたまりが枠で囲まれ動いた場所から ID の付いた霧が立ちのぼる。動きが強いほど青いグリッチが走り新しい点や霧の粒が音で鳴る。画面をタップすると UI が消える。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F117" s="6" t="n"/>
@@ -5593,10 +5593,41 @@
         </is>
       </c>
     </row>
+    <row r="118" ht="30" customHeight="1">
+      <c r="A118" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>SEIRETSU</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>映った人がピクセルソートのグリッチアートになる。動いたところが動いた向きに明るさ順で並べ替えられ光の筋になって尾を引き止まると明るいところが垂れていく。跳ぶかタップすると体ごと滝のように流れ落ちる。SILVER・SODIUM・PAPER・COLOR の四つの版。はじめは普通のカメラでボタンを押すと画面が一行ずつ並べ替えられて切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F118" s="6" t="n"/>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G117"/>
+  <autoFilter ref="A1:G118"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5717,6 +5748,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5863,7 +5895,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$117,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$118,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5886,7 +5918,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$117,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$118,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5909,7 +5941,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$117,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$118,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5930,7 +5962,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
AFTERIMAGE: add the owner's time-echo piece to the gallery
Owner-supplied file (アパート / APARTMENT); mechanism, shaders, palette and
sound kept as designed. Start screen aligned with the gallery (model and
camera pickers dropped: full-body model, front camera by default), plus
⟲ カメラ, a ⚙-hidden panel, the standard camera-failure message, and
snapshot/recording with the piece's own audio.
Adds the card, works.csv row, xlsx rebuild and register entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjAYv9LVh6abRGkArBYfFq
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5547,12 +5547,12 @@
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>KOGASHI</t>
+          <t>AFTERIMAGE</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t>映った人が映写機にかかった温黒調の古いフィルムになる。動いたところからフィルムが焦げて泡立ち琥珀色の縁をつれて白く焼け抜けやがて冷えて閉じる。すばやく動くとコマが滑りタップした場所に火が入る。PRINT・NITRATE・EKTA の三つのフィルム。はじめは普通のカメラでボタンを押すと映写機のランプが瞬いてコマが降りてくる。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだ作品。動くたびに少し前の自分が後ろへ一列に並び遠近で縮みながら光る縁をつれて墨色に沈み溶けていく。動いたところは白く光って光の粒と煙が立ちのぼり動きが鐘とノイズの音になる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F116" s="6" t="n"/>
@@ -5578,12 +5578,12 @@
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>MIST TRACKER</t>
+          <t>KOGASHI</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t>オーナーが持ち込んだ作品。カメラに映った動きに J0925 のような追跡 ID が次々に振られ点どうしが線で結ばれ動いたかたまりが枠で囲まれ動いた場所から ID の付いた霧が立ちのぼる。動きが強いほど青いグリッチが走り新しい点や霧の粒が音で鳴る。画面をタップすると UI が消える。撮影と録画ができる。</t>
+          <t>映った人が映写機にかかった温黒調の古いフィルムになる。動いたところからフィルムが焦げて泡立ち琥珀色の縁をつれて白く焼け抜けやがて冷えて閉じる。すばやく動くとコマが滑りタップした場所に火が入る。PRINT・NITRATE・EKTA の三つのフィルム。はじめは普通のカメラでボタンを押すと映写機のランプが瞬いてコマが降りてくる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F117" s="6" t="n"/>
@@ -5609,12 +5609,12 @@
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>SEIRETSU</t>
+          <t>MIST TRACKER</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t>映った人がピクセルソートのグリッチアートになる。動いたところが動いた向きに明るさ順で並べ替えられ光の筋になって尾を引き止まると明るいところが垂れていく。跳ぶかタップすると体ごと滝のように流れ落ちる。SILVER・SODIUM・PAPER・COLOR の四つの版。はじめは普通のカメラでボタンを押すと画面が一行ずつ並べ替えられて切り替わる。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだ作品。カメラに映った動きに J0925 のような追跡 ID が次々に振られ点どうしが線で結ばれ動いたかたまりが枠で囲まれ動いた場所から ID の付いた霧が立ちのぼる。動きが強いほど青いグリッチが走り新しい点や霧の粒が音で鳴る。画面をタップすると UI が消える。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F118" s="6" t="n"/>
@@ -5624,10 +5624,41 @@
         </is>
       </c>
     </row>
+    <row r="119" ht="30" customHeight="1">
+      <c r="A119" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>SEIRETSU</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>映った人がピクセルソートのグリッチアートになる。動いたところが動いた向きに明るさ順で並べ替えられ光の筋になって尾を引き止まると明るいところが垂れていく。跳ぶかタップすると体ごと滝のように流れ落ちる。SILVER・SODIUM・PAPER・COLOR の四つの版。はじめは普通のカメラでボタンを押すと画面が一行ずつ並べ替えられて切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="n"/>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G118"/>
+  <autoFilter ref="A1:G119"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5749,6 +5780,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5895,7 +5927,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$118,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$119,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5918,7 +5950,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$118,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$119,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5941,7 +5973,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$118,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$119,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5962,7 +5994,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
DENKOU: the head becomes a chrome helmet with an LED visor that mirrors your face
Black glass visor with an LED matrix that shows your blinks, gaze, mouth and
voice; head turns leave light trails, a held wink sweeps light across the shell.
SILVER / GOLD / NOIR finishes, a second person gets the next finish.
Plain camera ⇄ effect switch: blackout, the helmet drops on, LEDs boot.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011EBsBLAanhW4fDJd1B7BSN
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$120</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5655,10 +5655,41 @@
         </is>
       </c>
     </row>
+    <row r="120" ht="30" customHeight="1">
+      <c r="A120" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>DENKOU</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>頭がクロームのヘルメットになり黒いバイザーの LED があなたのまばたき・視線・口・声をそのまま映す。首を振ると LED の光が尾を引きウインクすると光がヘルメットをなでる。二人で映ると銀と金の二人組に。はじめは普通のカメラでボタンを押すと暗転してヘルメットが降りてくる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F120" s="6" t="n"/>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G119"/>
+  <autoFilter ref="A1:G120"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5781,6 +5812,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5927,7 +5959,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$119,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$120,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5950,7 +5982,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$119,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$120,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -5973,7 +6005,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$119,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$120,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -5994,7 +6026,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
MABAYUI: a storm of press flashes relights you in hard black and white
Photographers' flashes pop above a blurred crowd in the foreground; each flash
freezes the frame as a hard-lit monochrome photo and throws a sharp shadow on
the seamless wall, its direction set by where the flash came from. Move, then
strike a pose and the whole crowd fires. PRESS / NIGHT / TUNGSTEN.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011EBsBLAanhW4fDJd1B7BSN
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5686,10 +5686,41 @@
         </is>
       </c>
     </row>
+    <row r="121" ht="30" customHeight="1">
+      <c r="A121" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>MABAYUI</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>明かりが落ちた撮影会場で手前に並ぶカメラマンたちのフラッシュがあなたを撮りまくる。光るたびに白黒の硬い写真のように一瞬が止まり光の来た向きで白い壁に影がくっきり落ちる。動いてから止まってポーズを決めると連写の嵐。タップした場所からも焚ける。PRESS・NIGHT・TUNGSTEN の三つの版。はじめは普通のカメラでボタンを押すと暗転して正面の一発で会場が現れる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="n"/>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G120"/>
+  <autoFilter ref="A1:G121"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5813,6 +5844,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5959,7 +5991,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$120,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$121,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -5982,7 +6014,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$120,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$121,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6005,7 +6037,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$120,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$121,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6026,7 +6058,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
MEDAKA: a school of medaka silhouettes circles faces and hands
Top-view medaka silhouettes with a bending spine school around each face
and hand, cast soft shadows, scatter when you move fast and gather at
tapped food. Count, speed, size and ring width are adjustable; black,
orange, white or mixed fish. UI matches TOKERU.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011EBsBLAanhW4fDJd1B7BSN
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$122</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5717,10 +5717,41 @@
         </is>
       </c>
     </row>
+    <row r="122" ht="30" customHeight="1">
+      <c r="A122" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>MEDAKA</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>オーナーの依頼で作った作品。めだかの群れのシルエットがカメラに映った顔や手のまわりを群れのままぐるぐる泳ぐ。顔や手を速く動かすと散ってまた戻ってくる。タップした場所にはえさが落ちて集まる。黒・緋・白・まぜるの四種類で数・速さ・大きさ・輪の広さを調整できる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="n"/>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G121"/>
+  <autoFilter ref="A1:G122"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5845,6 +5876,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId121"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5991,7 +6023,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$121,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$122,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6014,7 +6046,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$121,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$122,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6037,7 +6069,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$121,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$122,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6058,7 +6090,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
MUGEN: stand inside an infinity mirror room
A Kusama-style mirrored box: thousands of lanterns (foreground bokeh,
far points, reflections in a water floor) and a lattice of mirror
reflections of you receding to the vanishing point, alternately
flipped. Each reflection plays a frame from (mirrors crossed x lag)
ago, so movement ripples outward as a wave, with a light pulse and a
glass-bell echo running into the depth. Gold / Souls / Ice palettes,
a slow room-wide blackout breath, rim light on the cut-out, and a
plain-camera to room transition that ignites from near to far.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013tNaHK5gR29sFQtrZ2LKAk
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5748,10 +5748,41 @@
         </is>
       </c>
     </row>
+    <row r="123" ht="30" customHeight="1">
+      <c r="A123" s="2" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>MUGEN</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>鏡張りの暗い部屋に灯りが何千もともり映ったあなたが左右と奥の鏡に何百人も並んで闇の果てまで続く。遠くの映り込みほど遅れてついてくるので動くと列が波打ち光の波が奥へ走る。金・七色・氷の三つの灯り。ときどき灯りがすべて消えてまた灯る。はじめは普通のカメラでボタンを押すと暗転して手前から灯りがともる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="n"/>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G122"/>
+  <autoFilter ref="A1:G123"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5877,6 +5908,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId122"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6023,7 +6055,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$122,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$123,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6046,7 +6078,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$122,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$123,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6069,7 +6101,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$122,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$123,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6090,7 +6122,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
NORI: a black silhouette with a white earphone cord, cut to the beat
The silhouette-ad poster grammar (one flat colour, a pure black
figure, a white cord) without any branding. PoseLandmarker with
segmentation masks for up to two people: a crisp upsampled silhouette,
verlet-rope earphone cords pinned at the ears and the hand (or the
pocket) joined at a free Y, a built-in groove whose bar downbeats
hard-cut the ground colour with a small push-in, jump / tap / mic
onset cuts, darker-tone echoes when moving fast, and a mode switch
where the cords drop in from above.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013tNaHK5gR29sFQtrZ2LKAk
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5779,10 +5779,41 @@
         </is>
       </c>
     </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="A124" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>NORI</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>映った人が一色の地の上の真っ黒なシルエットになり耳から白いイヤホンのコードが垂れて手のプレーヤーへつながる。踊ればコードがしなって跳ね内蔵のビートの拍で地の色がばっさり切り替わる。跳ぶかタップしても替わり速く動くと一段暗い色の残像がついてくる。二人で映ればそれぞれにコード。はじめは普通のカメラでボタンを押すと影になりコードが空から落ちてくる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="n"/>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G123"/>
+  <autoFilter ref="A1:G124"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5909,6 +5940,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId123"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6055,7 +6087,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$123,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$124,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6078,7 +6110,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$123,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$124,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6101,7 +6133,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$123,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$124,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6122,7 +6154,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
HIKU: add the owner's fingertip-string piece to the gallery
Five invisible strings between matching fingertips of both hands; pulling
them smears the camera image along the strings like a datamosh, and the
string length sets the pitch. Mechanism, shaders, palette and sound are the
owner's. Added the gallery conventions: ⟲ カメラ, a ⚙ panel, a shot button,
REC-FIX recording, the standard camera-error text and landmark guards.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011EBsBLAanhW4fDJd1B7BSN
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5764,12 +5764,12 @@
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>MUGEN</t>
+          <t>HIKU</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>鏡張りの暗い部屋に灯りが何千もともり映ったあなたが左右と奥の鏡に何百人も並んで闇の果てまで続く。遠くの映り込みほど遅れてついてくるので動くと列が波打ち光の波が奥へ走る。金・七色・氷の三つの灯り。ときどき灯りがすべて消えてまた灯る。はじめは普通のカメラでボタンを押すと暗転して手前から灯りがともる。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだ作品。両手の同じ指どうしのあいだに見えない糸が五本張られあやとりのように引くとカメラの映像が糸に沿ってデータモッシュのように溶けて伸び色ずれをつれて垂れながら残る。糸が短いほど高い音が鳴り片手なら指先だけが溶ける。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F123" s="6" t="n"/>
@@ -5795,12 +5795,12 @@
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>NORI</t>
+          <t>MUGEN</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t>映った人が一色の地の上の真っ黒なシルエットになり耳から白いイヤホンのコードが垂れて手のプレーヤーへつながる。踊ればコードがしなって跳ね内蔵のビートの拍で地の色がばっさり切り替わる。跳ぶかタップしても替わり速く動くと一段暗い色の残像がついてくる。二人で映ればそれぞれにコード。はじめは普通のカメラでボタンを押すと影になりコードが空から落ちてくる。撮影と録画ができる。</t>
+          <t>鏡張りの暗い部屋に灯りが何千もともり映ったあなたが左右と奥の鏡に何百人も並んで闇の果てまで続く。遠くの映り込みほど遅れてついてくるので動くと列が波打ち光の波が奥へ走る。金・七色・氷の三つの灯り。ときどき灯りがすべて消えてまた灯る。はじめは普通のカメラでボタンを押すと暗転して手前から灯りがともる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F124" s="6" t="n"/>
@@ -5810,10 +5810,41 @@
         </is>
       </c>
     </row>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>NORI</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>映った人が一色の地の上の真っ黒なシルエットになり耳から白いイヤホンのコードが垂れて手のプレーヤーへつながる。踊ればコードがしなって跳ね内蔵のビートの拍で地の色がばっさり切り替わる。跳ぶかタップしても替わり速く動くと一段暗い色の残像がついてくる。二人で映ればそれぞれにコード。はじめは普通のカメラでボタンを押すと影になりコードが空から落ちてくる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="n"/>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G124"/>
+  <autoFilter ref="A1:G125"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5941,6 +5972,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId122"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId124"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6087,7 +6119,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$124,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$125,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6110,7 +6142,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$124,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$125,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6133,7 +6165,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$124,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$125,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6154,7 +6186,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KARA: the body becomes a 3D-printed lattice you can see through
New effect: wherever you move, the skin shell breaks away cell by cell and
reveals a white Voronoi lattice (limbs as cylinders, the head as a sphere that
turns with you), with the studio wall visible through the holes and light
leaking through them into the shadow. Tap a part to open it, or sweep the
whole body with the orange print-head laser. NYLON / CHROME / OBSIDIAN /
LUMEN, studio or the real room, two people, photo and video.

Adds the gallery card, works.csv row, xlsx rebuild and register entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UW5xbMjdxUYsmeS6Ays6KX
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G125"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5841,10 +5841,41 @@
         </is>
       </c>
     </row>
+    <row r="126" ht="30" customHeight="1">
+      <c r="A126" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>KARA</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>映った人の体が 3D プリントの白い格子になる。動いたところから肌の殻が一枚ずつはがれて落ち格子の穴から向こうの壁が透ける。止まればゆっくり戻る。体をタップするとそこだけ開き「全身」で橙のレーザーが頭から足まで走る。NYLON・CHROME・OBSIDIAN・LUMEN の四つの素材。はじめは普通のカメラでボタンを押すとレーザーが体をなぞって切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="n"/>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G125"/>
+  <autoFilter ref="A1:G126"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5973,6 +6004,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId122"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId123"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId125"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6119,7 +6151,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$125,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$126,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6142,7 +6174,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$125,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$126,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6165,7 +6197,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$125,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$126,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6186,7 +6218,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
FRINGE: add the owner's transparent-feather piece to the gallery
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5857,12 +5857,12 @@
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>KARA</t>
+          <t>FRINGE</t>
         </is>
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t>映った人の体が 3D プリントの白い格子になる。動いたところから肌の殻が一枚ずつはがれて落ち格子の穴から向こうの壁が透ける。止まればゆっくり戻る。体をタップするとそこだけ開き「全身」で橙のレーザーが頭から足まで走る。NYLON・CHROME・OBSIDIAN・LUMEN の四つの素材。はじめは普通のカメラでボタンを押すとレーザーが体をなぞって切り替わる。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだ作品。動いたところから透明な羽が生えて体にまとわりつき、景色をガラスのように曲げながら消えていく。羽には少し前の自分が映る。絹・葉・ガラスの三つの羽。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F126" s="6" t="n"/>
@@ -5872,10 +5872,41 @@
         </is>
       </c>
     </row>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>KARA</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>映った人の体が 3D プリントの白い格子になる。動いたところから肌の殻が一枚ずつはがれて落ち格子の穴から向こうの壁が透ける。止まればゆっくり戻る。体をタップするとそこだけ開き「全身」で橙のレーザーが頭から足まで走る。NYLON・CHROME・OBSIDIAN・LUMEN の四つの素材。はじめは普通のカメラでボタンを押すとレーザーが体をなぞって切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="n"/>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G126"/>
+  <autoFilter ref="A1:G127"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6005,6 +6036,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId123"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6151,7 +6183,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$126,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$127,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6174,7 +6206,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$126,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$127,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6197,7 +6229,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$126,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$127,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6218,7 +6250,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
SHABON: add the owner's pressable soap-bubble piece to the gallery
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5903,10 +5903,41 @@
         </is>
       </c>
     </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="A128" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>SHABON</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが持ち込んだ作品。カメラの景色の前に大きなシャボン玉が浮かび、指で押すとへこんでぷるんと戻る。虹色の膜が流れて景色が映り込む。外側をなぞると玉が動く。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="n"/>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G127"/>
+  <autoFilter ref="A1:G128"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6037,6 +6068,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6183,7 +6215,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$127,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$128,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6206,7 +6238,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$127,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$128,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6229,7 +6261,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$127,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$128,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6250,7 +6282,7 @@
         <v>23</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
CRYSTAL BELLOWS: add the owner's crystal accordion to the instrument shelf
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1143,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1905,10 +1905,41 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>CRYSTAL BELLOWS</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが持ち込んだ作品。目の前にガラスのクリスタルが浮かび、両手で挟んで広げる・縮めるとアコーディオンのふいごのように和音が鳴る。左右で和音、上下で明るさ、傾けで揺らぎ。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>楽器</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G24"/>
+  <autoFilter ref="A1:G25"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1936,6 +1967,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6211,7 +6243,7 @@
         <v/>
       </c>
       <c r="C15" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$24,"〇")</f>
+        <f>COUNTIF(楽器!$B$2:$B$25,"〇")</f>
         <v/>
       </c>
       <c r="D15" s="13">
@@ -6234,7 +6266,7 @@
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$24,"△")</f>
+        <f>COUNTIF(楽器!$B$2:$B$25,"△")</f>
         <v/>
       </c>
       <c r="D16" s="13">
@@ -6257,7 +6289,7 @@
         <v/>
       </c>
       <c r="C17" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$24,"×")</f>
+        <f>COUNTIF(楽器!$B$2:$B$25,"×")</f>
         <v/>
       </c>
       <c r="D17" s="13">
@@ -6279,7 +6311,7 @@
         <v>14</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
         <v>127</v>

</xml_diff>

<commit_message>
DENNOU: digitized onto a light grid (new effect)
A red laser scans you off the plain camera onto a TRON-style grid: your
body becomes a black light-suit with glowing seams and a cool-lit face,
twin light walls trail behind you and turn at right angles as you move
sideways, hands paint light ribbons, and a jump or a tap derezzes you
into tumbling voxels before a scan line rebuilds you. Four colourways,
two people split into two colours, photo + recording.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CLPn3njED7YCwEUghXr6Wa
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ゲーム" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="楽器" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="エフェクト" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="使い方" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ゲーム" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楽器" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="エフェクト" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$129</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G128"/>
+  <dimension ref="A1:G129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5966,10 +5966,41 @@
         </is>
       </c>
     </row>
+    <row r="129" ht="30" customHeight="1">
+      <c r="A129" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>DENNOU</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>レーザーに読み込まれて、あなたは光の格子の世界に立つ。体は光の線が走る黒いスーツに、顔は冷たい光に照らされる。横に動けば両脇の光の壁が直角に折れながら地平線へ伸び、手は光の帯を引き、跳ぶか体をタップすると光の立方体に砕けてまた組み上がる。USER・PROGRAM・ISO・1982 の四色、二人で映ると二色に分かれる。はじめは普通のカメラで、ボタンを押すと赤いレーザーが走って切り替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="n"/>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G128"/>
+  <autoFilter ref="A1:G129"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6101,6 +6132,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6247,7 +6279,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$128,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$129,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6270,7 +6302,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$128,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$129,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6293,7 +6325,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$128,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$129,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6314,7 +6346,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TSUMIKI: the camera picture becomes a diorama of stacked cubes
From the owner's reference reel: each cell of the picture is a cube placed
along its camera ray at a depth made from the person mask (rounded from
the outline), the hand landmarks and a top-is-farther prior, so far walls
break into sparse floating cubes. Pop-out transition from the plain
picture, spilling cubes on movement, tap waves, BLOCK/TOY/MONO styles.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ゲーム" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楽器" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="エフェクト" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ゲーム" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="楽器" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="エフェクト" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="使い方" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G129"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5997,10 +5997,41 @@
         </is>
       </c>
     </row>
+    <row r="130" ht="30" customHeight="1">
+      <c r="A130" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>TSUMIKI</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが見せてくれた動画から作った作品。カメラの景色が小さなキューブを積んだ立体の箱庭になる。人と手は手前に飛び出し、奥の壁はまばらなブロックになって宙に浮く。動くとブロックがこぼれ、たたくと波が走る。BLOCK・TOY・MONO の三つ。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="n"/>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G129"/>
+  <autoFilter ref="A1:G130"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6133,6 +6164,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId129"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6279,7 +6311,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$129,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$130,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6302,7 +6334,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$129,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$130,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6325,7 +6357,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$129,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$130,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6346,7 +6378,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TOUEI: real-time face projection mapping in a dark room
A projector is the only light. Five face programs (Noh mask, skull, ink
tears, wireframe, kabuki red) are mapped onto the face mesh; structured
light stripes bend over the body; moving fast makes the lagged projection
spill onto the wall behind. Gray-code calibration as the camera switch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AjKRVmhJgaMJCwMfkyTMtv
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G130"/>
+  <dimension ref="A1:G131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6028,10 +6028,41 @@
         </is>
       </c>
     </row>
+    <row r="131" ht="30" customHeight="1">
+      <c r="A131" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>TOUEI</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>暗い部屋で、プロジェクターの光だけがあなたを照らす。顔には白い面・骸骨・墨の涙・網・隈取りがぴたりと映り、体には光の縞が曲面に沿って走る。速く動くと光が追いつかず、顔の絵が奥の壁へこぼれる。首を横に振ると面が替わる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="n"/>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G130"/>
+  <autoFilter ref="A1:G131"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6165,6 +6196,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId130"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6311,7 +6343,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$130,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$131,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6334,7 +6366,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$130,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$131,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6357,7 +6389,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$130,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$131,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6378,7 +6410,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TSUMAMU: pinch the camera picture and pull it like a gel sheet
Thumb-and-index pinch grabs the image as an elastic membrane; release
springs back with a pitched boing; two hands stretch between them;
flicks send ripples. GEL / LATEX / HONEY materials.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AjKRVmhJgaMJCwMfkyTMtv
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$132</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:G132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6059,10 +6059,41 @@
         </is>
       </c>
     </row>
+    <row r="132" ht="30" customHeight="1">
+      <c r="A132" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>TSUMAMU</t>
+        </is>
+      </c>
+      <c r="E132" s="5" t="inlineStr">
+        <is>
+          <t>カメラの映像を親指と人差し指でつまんで引っぱれる。映像はゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、指ではじくと波紋が走る。ゼリー・ゴム・蜜の三つの素材。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F132" s="6" t="n"/>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G131"/>
+  <autoFilter ref="A1:G132"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6197,6 +6228,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId131"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6343,7 +6375,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$131,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$132,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6366,7 +6398,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$131,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$132,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6389,7 +6421,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$131,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$132,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6410,7 +6442,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TSUMAMU NAKED: keep the first version of TSUMAMU as its own piece
The state before colour modes, tearing, stickers and voice, with only
the plain-camera flatten fix applied.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AjKRVmhJgaMJCwMfkyTMtv
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G132"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6090,10 +6090,41 @@
         </is>
       </c>
     </row>
+    <row r="133" ht="30" customHeight="1">
+      <c r="A133" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>TSUMAMU NAKED</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>TSUMAMU の最初の版（色の切り替え・ちぎる・貼る・声を足す前）。カメラの映像を親指と人差し指でつまんで引っぱると、ゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、指ではじくと波紋が走る。ゼリー・ゴム・蜜の三つの素材。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F133" s="6" t="n"/>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G132"/>
+  <autoFilter ref="A1:G133"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6229,6 +6260,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId132"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6375,7 +6407,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$132,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$133,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6398,7 +6430,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$132,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$133,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6421,7 +6453,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$132,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$133,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6442,7 +6474,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
SHARD: add the owner's sample editor as an effect piece (to grow into video)
Owner-supplied shard.html, kept as-is apart from the gallery title,
description and art-direction header.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AjKRVmhJgaMJCwMfkyTMtv
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$134</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G133"/>
+  <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6044,12 +6044,12 @@
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>TOUEI</t>
+          <t>SHARD</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>暗い部屋で、プロジェクターの光だけがあなたを照らす。顔には白い面・骸骨・墨の涙・網・隈取りがぴたりと映り、体には光の縞が曲面に沿って走る。速く動くと光が追いつかず、顔の絵が奥の壁へこぼれる。首を横に振ると面が替わる。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだサンプルエディタ。録音ボタンを長押しして声や物音を録り、波形から好きな所を切り出して、右の線をなぞると音程を変えて弾ける。逆再生・正規化・自動トリム・音程の自動検出・フェード・WAV 保存。これから映像の作品に育てていく。</t>
         </is>
       </c>
       <c r="F131" s="6" t="n"/>
@@ -6075,12 +6075,12 @@
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>TSUMAMU</t>
+          <t>TOUEI</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>カメラの映像を指でつまんで引っぱれる（「手でつまむ」を入にすればカメラに映った親指と人差し指でも）。映像はゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、引っぱりすぎるとちぎれて、切れ端を好きな所にシールのように貼れる（「↺ リセット」でまとめて落とせる）。指ではじくと波紋が走り、声や手拍子でも膜が震える。ゼリー・ゴム・蜜の三つの素材と、素・銀・桃・藍・夜光の五つの色。撮影と録画ができる。</t>
+          <t>暗い部屋で、プロジェクターの光だけがあなたを照らす。顔には白い面・骸骨・墨の涙・網・隈取りがぴたりと映り、体には光の縞が曲面に沿って走る。速く動くと光が追いつかず、顔の絵が奥の壁へこぼれる。首を横に振ると面が替わる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F132" s="6" t="n"/>
@@ -6106,12 +6106,12 @@
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>TSUMAMU NAKED</t>
+          <t>TSUMAMU</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>TSUMAMU の最初の版（色の切り替え・ちぎる・貼る・声を足す前）。カメラの映像を親指と人差し指でつまんで引っぱると、ゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、指ではじくと波紋が走る。ゼリー・ゴム・蜜の三つの素材。撮影と録画ができる。</t>
+          <t>カメラの映像を指でつまんで引っぱれる（「手でつまむ」を入にすればカメラに映った親指と人差し指でも）。映像はゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、引っぱりすぎるとちぎれて、切れ端を好きな所にシールのように貼れる（「↺ リセット」でまとめて落とせる）。指ではじくと波紋が走り、声や手拍子でも膜が震える。ゼリー・ゴム・蜜の三つの素材と、素・銀・桃・藍・夜光の五つの色。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F133" s="6" t="n"/>
@@ -6121,10 +6121,41 @@
         </is>
       </c>
     </row>
+    <row r="134" ht="30" customHeight="1">
+      <c r="A134" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>TSUMAMU NAKED</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>TSUMAMU の最初の版（色の切り替え・ちぎる・貼る・声を足す前）。カメラの映像を親指と人差し指でつまんで引っぱると、ゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、指ではじくと波紋が走る。ゼリー・ゴム・蜜の三つの素材。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F134" s="6" t="n"/>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G133"/>
+  <autoFilter ref="A1:G134"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6261,6 +6292,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId133"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6407,7 +6439,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$133,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$134,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6430,7 +6462,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$133,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$134,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6453,7 +6485,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$133,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$134,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6474,7 +6506,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
GEKIGA CAM: add the owner's retro gekiga comic camera
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6044,12 +6044,12 @@
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>SHARD</t>
+          <t>GEKIGA CAM</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>オーナーが持ち込んだサンプルエディタ。録音ボタンを長押しして声や物音を録り、波形から好きな所を切り出して、右の線をなぞると音程を変えて弾ける。逆再生・正規化・自動トリム・音程の自動検出・フェード・WAV 保存。これから映像の作品に育てていく。</t>
+          <t>オーナーが持ち込んだ作品。カメラの映像がそのまま昔の劇画の一コマになる。平らに塗られた面と墨の輪郭線とべた塗りの影、染みと焼けのある紙、ちぎれた紙のふち。劇画セピア・浮世絵・墨・夕焼け・ポップの五つ。写真と動画で撮れる。</t>
         </is>
       </c>
       <c r="F131" s="6" t="n"/>
@@ -6075,12 +6075,12 @@
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>TOUEI</t>
+          <t>SHARD</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>暗い部屋で、プロジェクターの光だけがあなたを照らす。顔には白い面・骸骨・墨の涙・網・隈取りがぴたりと映り、体には光の縞が曲面に沿って走る。速く動くと光が追いつかず、顔の絵が奥の壁へこぼれる。首を横に振ると面が替わる。撮影と録画ができる。</t>
+          <t>オーナーが持ち込んだサンプルエディタ。録音ボタンを長押しして声や物音を録り、波形から好きな所を切り出して、右の線をなぞると音程を変えて弾ける。逆再生・正規化・自動トリム・音程の自動検出・フェード・WAV 保存。これから映像の作品に育てていく。</t>
         </is>
       </c>
       <c r="F132" s="6" t="n"/>
@@ -6106,12 +6106,12 @@
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>TSUMAMU</t>
+          <t>TOUEI</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>カメラの映像を指でつまんで引っぱれる（「手でつまむ」を入にすればカメラに映った親指と人差し指でも）。映像はゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、引っぱりすぎるとちぎれて、切れ端を好きな所にシールのように貼れる（「↺ リセット」でまとめて落とせる）。指ではじくと波紋が走り、声や手拍子でも膜が震える。ゼリー・ゴム・蜜の三つの素材と、素・銀・桃・藍・夜光の五つの色。撮影と録画ができる。</t>
+          <t>暗い部屋で、プロジェクターの光だけがあなたを照らす。顔には白い面・骸骨・墨の涙・網・隈取りがぴたりと映り、体には光の縞が曲面に沿って走る。速く動くと光が追いつかず、顔の絵が奥の壁へこぼれる。首を横に振ると面が替わる。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F133" s="6" t="n"/>
@@ -6137,12 +6137,12 @@
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>TSUMAMU NAKED</t>
+          <t>TSUMAMU</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>TSUMAMU の最初の版（色の切り替え・ちぎる・貼る・声を足す前）。カメラの映像を親指と人差し指でつまんで引っぱると、ゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、指ではじくと波紋が走る。ゼリー・ゴム・蜜の三つの素材。撮影と録画ができる。</t>
+          <t>カメラの映像を指でつまんで引っぱれる（「手でつまむ」を入にすればカメラに映った親指と人差し指でも）。映像はゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、引っぱりすぎるとちぎれて、切れ端を好きな所にシールのように貼れる（「↺ リセット」でまとめて落とせる）。指ではじくと波紋が走り、声や手拍子でも膜が震える。ゼリー・ゴム・蜜の三つの素材と、素・銀・桃・藍・夜光の五つの色。撮影と録画ができる。</t>
         </is>
       </c>
       <c r="F134" s="6" t="n"/>
@@ -6152,10 +6152,41 @@
         </is>
       </c>
     </row>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>TSUMAMU NAKED</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>TSUMAMU の最初の版（色の切り替え・ちぎる・貼る・声を足す前）。カメラの映像を親指と人差し指でつまんで引っぱると、ゼリーのような透明な膜になって伸び、離すとぷるんと揺れて「ぼよん」と鳴りながら戻る。両手でつまめば手のあいだで引き伸ばせ、指ではじくと波紋が走る。ゼリー・ゴム・蜜の三つの素材。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="n"/>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G134"/>
+  <autoFilter ref="A1:G135"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6293,6 +6324,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId134"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6439,7 +6471,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$134,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$135,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6462,7 +6494,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$134,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$135,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6485,7 +6517,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$134,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$135,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6506,7 +6538,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TATAMU: fold the room like paper with your hand
Bend your fingers and the picture folds along your knuckles, the outer
part rising toward you and over your head (the Paris street in Inception).
Two hands raise both walls; tap to keep a crease and build a box.
Under the lifted paper, you from two seconds ago on a darker level.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DugDKQLptTcGToTXPD8zk9
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$136</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G135"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6183,10 +6183,41 @@
         </is>
       </c>
     </row>
+    <row r="136" ht="30" customHeight="1">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>TATAMU</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>指を曲げると指の付け根の線で部屋の景色が紙のように折れて起き上がり頭上へ覆いかぶさる。両手なら両側の壁が立ちタップで折り目を残して部屋を箱のように組める。</t>
+        </is>
+      </c>
+      <c r="F136" s="6" t="n"/>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G135"/>
+  <autoFilter ref="A1:G136"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6325,6 +6356,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId135"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6471,7 +6503,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$135,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$136,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6494,7 +6526,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$135,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$136,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6517,7 +6549,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$135,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$136,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6538,7 +6570,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
PSYCHE MIRROR II: stare and your hair bursts into liquid marbled paint
A new version of PSYCHE MIRROR built from the owner's three references
(MINIMA's paint-haired portrait, a holi powder burst, a neon splatter).
Hair becomes advected marbling paint, the face turns into a white paper
poster, powder explodes behind the head and droplets fly with trails.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6199,12 +6199,12 @@
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>TATAMU</t>
+          <t>PSYCHE MIRROR II</t>
         </is>
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t>指を曲げると指の付け根の線で部屋の景色が紙のように折れて起き上がり頭上へ覆いかぶさる。両手なら両側の壁が立ちタップで折り目を残して部屋を箱のように組める。</t>
+          <t>PSYCHE MIRROR の新しい版。カメラをじっと見つめると髪が液体のマーブル絵の具になって頭からはじけ出す。顔は白い紙のように抜け後ろで色の粉が爆発ししぶきが線を引いて飛ぶ。頭をふるとしぶき・口をあけると爆発・目を長めにとじると配色がかわる。</t>
         </is>
       </c>
       <c r="F136" s="6" t="n"/>
@@ -6214,10 +6214,41 @@
         </is>
       </c>
     </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>TATAMU</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>指を曲げると指の付け根の線で部屋の景色が紙のように折れて起き上がり頭上へ覆いかぶさる。両手なら両側の壁が立ちタップで折り目を残して部屋を箱のように組める。</t>
+        </is>
+      </c>
+      <c r="F137" s="6" t="n"/>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G136"/>
+  <autoFilter ref="A1:G137"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6357,6 +6388,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId136"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6503,7 +6535,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$136,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$137,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6526,7 +6558,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$136,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$137,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6549,7 +6581,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$136,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$137,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6570,7 +6602,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TAMASUDARE: reach through a curtain of glass beads
A bead curtain hangs in front of the camera. Hands and forearms part the
strands, a fist gathers a bunch, a fast swipe flings them, and every bead
shows the room upside down like a tiny lens. Four bead types.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$138</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6245,10 +6245,41 @@
         </is>
       </c>
     </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>TAMASUDARE</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>カメラの前に硝子の玉すだれが下りてくる。手や腕を入れると玉がよけて揺れからからと鳴る。握れば玉の束をつかんで寄せられはなせば揺れもどる。玉はひとつずつ向こうの景色をさかさまに映す。クリスタル・オーロラ・琥珀・黒硝子の四つ。</t>
+        </is>
+      </c>
+      <c r="F138" s="6" t="n"/>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G137"/>
+  <autoFilter ref="A1:G138"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6389,6 +6420,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId137"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6535,7 +6567,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$137,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$138,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6558,7 +6590,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$137,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$138,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6581,7 +6613,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$137,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$138,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6602,7 +6634,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
SHIPPAN: the camera becomes a wet-plate camera
A tintype portrait studio. One plate rests on black velvet: the sitter is
lit by a window light in front of a dark mottled backdrop, the eyes are
sharp and the rest swirls like a Petzval lens, and the image sinks into
black at the hand-poured edge of the coat. Hold still for three seconds
and the developer brings up a pale negative on the cream plate, then the
fixer runs down and turns it into a positive on the black. Four plates:
ferrotype, ambrotype, ruby ambrotype, daguerreotype (tilt it and it turns
negative like a mirror).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$139</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6261,12 +6261,12 @@
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>TAMASUDARE</t>
+          <t>SHIPPAN</t>
         </is>
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>カメラの前に硝子の玉すだれが下りてくる。手や腕を入れると玉がよけて揺れからからと鳴る。握れば玉の束をつかんで寄せられはなせば揺れもどる。玉はひとつずつ向こうの景色をさかさまに映す。クリスタル・オーロラ・琥珀・黒硝子の四つ。</t>
+          <t>カメラが百五十年前の湿板写真機になる。黒い板に窓の光を受けた銀色の肖像が浮かびまわりは渦を巻いてぼける。三秒じっとするとクリーム色の板に陰画が浮かび定着液が流れて黒地の陽画に変わる。鉄板・硝子板・紅硝子・銀板の四つ。</t>
         </is>
       </c>
       <c r="F138" s="6" t="n"/>
@@ -6276,10 +6276,41 @@
         </is>
       </c>
     </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>TAMASUDARE</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>カメラの前に硝子の玉すだれが下りてくる。手や腕を入れると玉がよけて揺れからからと鳴る。握れば玉の束をつかんで寄せられはなせば揺れもどる。玉はひとつずつ向こうの景色をさかさまに映す。クリスタル・オーロラ・琥珀・黒硝子の四つ。</t>
+        </is>
+      </c>
+      <c r="F139" s="6" t="n"/>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G138"/>
+  <autoFilter ref="A1:G139"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6421,6 +6452,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6567,7 +6599,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$138,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$139,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6590,7 +6622,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$138,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$139,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6613,7 +6645,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$138,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$139,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6634,7 +6666,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
SAKEME: slash the red canvas you are standing behind
The screen becomes one red canvas and you are behind it. Your body leans
on the cloth as a soft relief and your hand presses it finger by finger.
Swipe a hand fast and the index fingertip cuts a Fontana slit: it springs
open behind the blade, the lips curl back into the dark, and you peek
through. Re-stretch rolls a fresh canvas down with stapler clicks. Four
canvases: red, white, black, ultramarine.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6307,10 +6307,41 @@
         </is>
       </c>
     </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>SAKEME</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>画面が一枚の真っ赤なキャンバスになりあなたはその裏側にいる。体と手が布を押すとその形が浮き彫りになり手をすばやく払うとフォンタナの絵のように切れ目が入る。めくれた縁の奥の暗がりからあなたがのぞく。赤・白・黒・群青の四つ。</t>
+        </is>
+      </c>
+      <c r="F140" s="6" t="n"/>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G139"/>
+  <autoFilter ref="A1:G140"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6453,6 +6484,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId137"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6599,7 +6631,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$139,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$140,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6622,7 +6654,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$139,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$140,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6645,7 +6677,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$139,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$140,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6666,7 +6698,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KOUGA: draw lines of light in the air, frozen by one strobe (after Gjon Mili, 1949)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D2Nuw72YHWHVKD97o5iL9T
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6338,10 +6338,41 @@
         </is>
       </c>
     </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>KOUGA</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>灯りを消した部屋で人差し指を立てると指先が空中に光の線を描く。止まってポーズを決めるとストロボが焚かれ銀塩写真のあなたが光の線の中に焼き付く。描くのをやめると線がゆっくり回る。1949・EKTA・CYANO・SAFELIGHT の四つ。はじめは普通のカメラでボタンを押すと白熱灯が赤く落ちてストロボ一発で現れる。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F141" s="6" t="n"/>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G140"/>
+  <autoFilter ref="A1:G141"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6485,6 +6516,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId137"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6631,7 +6663,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$140,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$141,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6654,7 +6686,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$140,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$141,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6677,7 +6709,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$140,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$141,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6698,7 +6730,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
TOGE: black ferrofluid rises in spikes toward your hand
The screen becomes the surface of a black liquid seen from above, and you
are dimly reflected in it. A hand coming closer to the screen is a magnet:
the liquid gathers into a low mound and hundreds of glossy needles stand
up and lean toward the palm, following it as it moves. Pull away and the
mound collapses, and the ripples warp your reflected face. Four lights:
void, red, gold, blue. After Sachiko Kodama's ferrofluid sculptures and
Caravaggio's Narcissus.

CLAUDE.md: the owner asked what was fun about SAKEME; looking stylish is
not enough, the piece has to be fun to touch too.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6369,10 +6369,41 @@
         </is>
       </c>
     </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>TOGE</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>画面が黒い液体の水面になりあなたはそこにほの暗く映る。手を画面に近づけると磁性流体が何百本もの棘になって手のひらへ立ち上がり手を追ってついてくる。離すと山がくずれて映ったあなたの顔が波紋にゆがむ。虚空・紅・金・青の四つ。</t>
+        </is>
+      </c>
+      <c r="F142" s="6" t="n"/>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G141"/>
+  <autoFilter ref="A1:G142"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6517,6 +6548,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId141"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6663,7 +6695,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$141,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$142,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6686,7 +6718,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$141,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$142,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6709,7 +6741,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$141,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$142,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6730,7 +6762,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
AMAYADORI: backlit rain that stops above you (after Rain Room)
A black room lit by one lamp behind; silver rain in three depths stops on an
invisible umbrella just above your head and shoulders, and the spray draws
your outline in light. The sensor lags, so moving fast gets you wet; tap to
stop the drops in mid-air and walk through them. Four lamps (BARBICAN,
SODIUM, NOIR, CRIMSON), a ceiling mode that dries the whole column as in the
real installation, and a lights-out / lamp-strike / rain-front transition.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V9vL2QMb1xLmGcE2mcpPGn
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$143</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:G143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6400,10 +6400,41 @@
         </is>
       </c>
     </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>AMAYADORI</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>暗い部屋にうしろから一灯の光が差し光る雨が降りつづける。あなたの頭と肩の上でだけ雨がやみしぶきが輪郭を光でなぞる。手をのばせばその上でもやみすばやく動くと間に合わない雨粒があなたを濡らす。タップすると雨粒が宙で止まる。BARBICAN・SODIUM・NOIR・CRIMSON の四つ。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F143" s="6" t="n"/>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G142"/>
+  <autoFilter ref="A1:G143"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6549,6 +6580,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId142"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6695,7 +6727,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$142,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$143,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6718,7 +6750,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$142,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$143,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6741,7 +6773,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$142,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$143,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6762,7 +6794,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
RAINBOW FLOW: add the owner's rainbow fluid piece to the gallery
Move a hand in front of the camera and rainbow liquid pours from the
fingers; the liquid shines like chrome, bends the scene behind it, and the
hand stays in front of it. Mechanism, shaders, colours and UI are the
owner's. Added the gallery conventions: REC-FIX and RESUME-FIX, title and
description, ⟲ カメラ, a shot button and recording, the standard
camera-error text, and landmark guards.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$144</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6431,10 +6431,41 @@
         </is>
       </c>
     </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>RAINBOW FLOW</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが持ち込んだ作品。カメラの前で手を動かすと指先から虹色の液体があふれ出す。液体はクロームのように光ってうしろの景色をゆがめ手は液体の手前に見える。虹・炎・オーロラ・単色の四つ。</t>
+        </is>
+      </c>
+      <c r="F144" s="6" t="n"/>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G143"/>
+  <autoFilter ref="A1:G144"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6581,6 +6612,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId141"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId143"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6727,7 +6759,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$143,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$144,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6750,7 +6782,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$143,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$144,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6773,7 +6805,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$143,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$144,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6794,7 +6826,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
PROFILE MASK: add the owner's profile-mask illusion piece to the gallery
Take one side-view photo; facing the camera, a white board covers the
screen and a window cut in the shape of your profile follows your face,
so the outline reads as a profile and the inside as a front face.

The owner's mechanism, screens and wording are kept. Added for the
gallery: REC-FIX and RESUME-FIX, the title and description, the
⟲ カメラ button, a still shot button, the standard camera error text,
face landmark guards, recovery when switching cameras fails, and a
visible message when the models fail to load. The header is tightened
on narrow phones so ⟲ カメラ stays on screen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$145</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G144"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6447,12 +6447,12 @@
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>RAINBOW FLOW</t>
+          <t>PROFILE MASK</t>
         </is>
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>オーナーが持ち込んだ作品。カメラの前で手を動かすと指先から虹色の液体があふれ出す。液体はクロームのように光ってうしろの景色をゆがめ手は液体の手前に見える。虹・炎・オーロラ・単色の四つ。</t>
+          <t>オーナーが持ち込んだ作品。横を向いて横顔を1枚撮ってから正面を向くとまわりが白い板でふさがれ自分の横顔の形の窓から正面の顔がのぞく。輪郭は横顔で中身は正面顔の騙し絵。しゃべると窓のあごも動きそのまま録画できる。</t>
         </is>
       </c>
       <c r="F144" s="6" t="n"/>
@@ -6462,10 +6462,41 @@
         </is>
       </c>
     </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="inlineStr">
+        <is>
+          <t>RAINBOW FLOW</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが持ち込んだ作品。カメラの前で手を動かすと指先から虹色の液体があふれ出す。液体はクロームのように光ってうしろの景色をゆがめ手は液体の手前に見える。虹・炎・オーロラ・単色の四つ。</t>
+        </is>
+      </c>
+      <c r="F145" s="6" t="n"/>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G144"/>
+  <autoFilter ref="A1:G145"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6613,6 +6644,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId141"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId144"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6759,7 +6791,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$144,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$145,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6782,7 +6814,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$144,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$145,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6805,7 +6837,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$144,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$145,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6826,7 +6858,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
KARAKURI: a kinetic wooden mirror after Daniel Rozin
Over a thousand small tiles on a framed panel in a dark gallery tilt one
by one under a single spotlight, and their shading draws the viewer's
portrait. Servo lag makes movement ripple across the wall, fast motion
flips tiles to their bright backs, and the portrait lets go tile by tile
when the person leaves. Four materials: walnut, brass, urushi, ash.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163rgqPhLvrpoxCg6NthKJD
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$146</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6493,10 +6493,41 @@
         </is>
       </c>
     </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>KARAKURI</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>明かりの落ちた美術館の壁で千枚あまりの木の小板が一枚ずつ傾き上からの一灯の陰影であなたの肖像を描く。動けば板が波打って鳴り速く動くと裏返り立ち去ると形が一枚ずつほどける。画面をたたくとそこから板がめくれる。胡桃・真鍮・黒漆・タモの四つ。撮影と録画ができる。</t>
+        </is>
+      </c>
+      <c r="F146" s="6" t="n"/>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G145"/>
+  <autoFilter ref="A1:G146"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6645,6 +6676,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId145"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6791,7 +6823,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$145,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$146,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6814,7 +6846,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$145,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$146,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6837,7 +6869,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$145,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$146,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6858,7 +6890,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
USUBA: add the owner's glass-blade piece to the gallery
Moving a hand sheds hundreds of thin glass blades from the fingers and
the edge of the hand; they trail behind the motion, split the picture
into magenta and green by refraction, then hang and sink once the hand
leaves. The owner's file already met the gallery rules (REC-FIX,
RESUME-FIX, ⟲ カメラ, the standard camera error text, landmark
guards, shot and recording), so it is added unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G146"/>
+  <dimension ref="A1:G147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6524,10 +6524,41 @@
         </is>
       </c>
     </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="A147" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>USUBA</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが持ち込んだ作品。手を動かすと指と手の縁から硝子の薄刃が何百枚もこぼれ動いた向きの後ろへなびく。刃の中では映像が引き伸ばされ屈折で赤紫と黄緑に割れる。手が去ると刃は垂れ下がりゆっくり沈んで消える。</t>
+        </is>
+      </c>
+      <c r="F147" s="6" t="n"/>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G146"/>
+  <autoFilter ref="A1:G147"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6677,6 +6708,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId146"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6823,7 +6855,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$146,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$147,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6846,7 +6878,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$146,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$147,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6869,7 +6901,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$146,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$147,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6890,7 +6922,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>

<commit_message>
MOYA: add the owner's face-melting fluid camera to the gallery
The camera finds a face (or, with no one in frame, one object) and
stirs just that area like smoke or liquid, with rainbow-split edges.
The owner's mechanism, shaders, screens and wording are kept. Added for
the gallery: REC-FIX and RESUME-FIX, the title and description, the
⟲ カメラ label, a REC button, the standard camera error text, recovery
when switching cameras fails, and checks on the detection boxes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tcgSewXTZavwZExmC5gj3
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$148</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1980,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G147"/>
+  <dimension ref="A1:G148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6555,10 +6555,41 @@
         </is>
       </c>
     </row>
+    <row r="148" ht="30" customHeight="1">
+      <c r="A148" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>MOYA</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="inlineStr">
+        <is>
+          <t>オーナーが持ち込んだ作品。カメラに写った人の顔を見つけてそこだけを煙や液体のようにかき混ぜて溶かす。人がいないときは写っている物をひとつ選んで溶かしうねりの縁は虹色に割れる。顔だけ・物だけ・タップでも選べる。</t>
+        </is>
+      </c>
+      <c r="F148" s="6" t="n"/>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G147"/>
+  <autoFilter ref="A1:G148"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6709,6 +6740,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId145"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="rId147"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -6855,7 +6887,7 @@
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$147,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$148,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -6878,7 +6910,7 @@
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$147,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$148,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -6901,7 +6933,7 @@
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$147,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$148,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -6922,7 +6954,7 @@
         <v>24</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>